<commit_message>
ID-56: Add v2.2.1 Claim Update scenario tests (Client and Server suites) (#74)
* Add Claim Update test group for PAS server v2.2.1 validation

* Correct typo in session_endpoint_url method name and update all references

* Add requirement coverage for PAS v2.2.1 and update test suite generator templates

* update requirements files

* Refactor Claim Update workflow tests into modular test classes and add support for cancel-entire-request validation

* Append "See Messages for details" to Claim Update workflow assertion error messages

* Update requirements coverage and link v2.2.1 PAS claim update tests to profile-based requirements.

---------

Co-authored-by: Karl Naden <karl@glenviewassociates.com>
</commit_message>
<xml_diff>
--- a/lib/davinci_pas_test_kit/requirements/hl7.fhir.us.davinci-pas_2.2.1_requirements.xlsx
+++ b/lib/davinci_pas_test_kit/requirements/hl7.fhir.us.davinci-pas_2.2.1_requirements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karlnaden/GlenViewAssociates/Inferno/source/davinci-pas-test-kit/lib/davinci_pas_test_kit/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BE8ABAA-F3C4-8A43-9C59-A898033B7FFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B3BEC42-E831-164D-B0D3-5BF7C2F1422B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20100" activeTab="1" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="767" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="449">
   <si>
     <r>
       <rPr>
@@ -2703,42 +2703,42 @@
     <t>Attestation</t>
   </si>
   <si>
-    <t>TODO - adjust MS tests</t>
-  </si>
-  <si>
     <t>Attestation (maybe Mechanical piece- require incomplete responses - should happen naturally)</t>
-  </si>
-  <si>
-    <t>TODO</t>
-  </si>
-  <si>
-    <t>TODO - see CRD ID-119</t>
-  </si>
-  <si>
-    <t>TODO - update scenario</t>
-  </si>
-  <si>
-    <t>TODO - check US Core logic</t>
-  </si>
-  <si>
-    <t>Attestatation</t>
-  </si>
-  <si>
-    <t>Done?</t>
-  </si>
-  <si>
-    <t>Wrong Actor</t>
-  </si>
-  <si>
-    <t>?? Mechnical if possible</t>
-  </si>
-  <si>
-    <t>Wrong Actor - Mechnical</t>
   </si>
   <si>
     <t>Bundle.entry.fullUrl values **SHALL** be:
 - the URL at which the resource is available from the EHR if exposed via the client's REST interface; or
 - the form "urn:uuid:[some guid]"</t>
+  </si>
+  <si>
+    <t>ID-148</t>
+  </si>
+  <si>
+    <t>ID-150</t>
+  </si>
+  <si>
+    <t>Future</t>
+  </si>
+  <si>
+    <t>ID-56</t>
+  </si>
+  <si>
+    <t>Done - Double Check</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>ID-151</t>
+  </si>
+  <si>
+    <t>Actor adjusted payer -&gt; client</t>
+  </si>
+  <si>
+    <t>Actor adjusted client -&gt; payer</t>
+  </si>
+  <si>
+    <t>Actor adjusted client + payer -&gt; payer</t>
   </si>
 </sst>
 </file>
@@ -3138,7 +3138,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3155,7 +3155,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -3596,72 +3595,72 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="133.5" style="24" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" style="20"/>
-    <col min="3" max="3" width="91.1640625" style="20" customWidth="1"/>
-    <col min="4" max="16384" width="10.83203125" style="15"/>
+    <col min="1" max="1" width="133.5" style="23" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" style="19"/>
+    <col min="3" max="3" width="91.1640625" style="19" customWidth="1"/>
+    <col min="4" max="16384" width="10.83203125" style="14"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="340" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="25" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="33" t="s">
+      <c r="A1" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="32" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="124.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="37"/>
+      <c r="C2" s="36"/>
     </row>
     <row r="3" spans="1:3" ht="134" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="34"/>
+      <c r="C3" s="33"/>
     </row>
     <row r="4" spans="1:3" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="44" t="s">
         <v>69</v>
       </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="36"/>
+      <c r="B4" s="34"/>
+      <c r="C4" s="35"/>
     </row>
     <row r="5" spans="1:3" ht="258" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="46"/>
-      <c r="B5" s="39"/>
-      <c r="C5" s="34"/>
+      <c r="A5" s="45"/>
+      <c r="B5" s="38"/>
+      <c r="C5" s="33"/>
     </row>
     <row r="6" spans="1:3" ht="164" x14ac:dyDescent="0.2">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="27"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="26"/>
     </row>
     <row r="7" spans="1:3" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="47" t="s">
+      <c r="A7" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="48"/>
+      <c r="B7" s="47"/>
     </row>
     <row r="8" spans="1:3" ht="126" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="47"/>
-      <c r="B8" s="49"/>
+      <c r="A8" s="46"/>
+      <c r="B8" s="48"/>
     </row>
     <row r="9" spans="1:3" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="45"/>
-      <c r="B9" s="38"/>
+      <c r="A9" s="44"/>
+      <c r="B9" s="37"/>
     </row>
     <row r="10" spans="1:3" ht="292" x14ac:dyDescent="0.2">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="21" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="23"/>
+      <c r="A11" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3684,19 +3683,19 @@
     <col min="5" max="5" width="10.83203125" style="7"/>
     <col min="6" max="6" width="13.33203125" style="8" customWidth="1"/>
     <col min="7" max="7" width="14" style="7" customWidth="1"/>
-    <col min="8" max="8" width="24.6640625" style="16" customWidth="1"/>
-    <col min="9" max="9" width="10" style="30" customWidth="1"/>
-    <col min="10" max="10" width="22" style="30" customWidth="1"/>
-    <col min="11" max="11" width="10.5" style="30" customWidth="1"/>
-    <col min="12" max="12" width="25.83203125" style="30" customWidth="1"/>
+    <col min="8" max="8" width="24.6640625" style="15" customWidth="1"/>
+    <col min="9" max="9" width="10" style="29" customWidth="1"/>
+    <col min="10" max="10" width="22" style="29" customWidth="1"/>
+    <col min="11" max="11" width="10.5" style="29" customWidth="1"/>
+    <col min="12" max="12" width="25.83203125" style="29" customWidth="1"/>
     <col min="13" max="13" width="20" style="9" customWidth="1"/>
     <col min="14" max="14" width="28.5" style="9" customWidth="1"/>
     <col min="15" max="16" width="10.83203125" style="10" customWidth="1"/>
-    <col min="17" max="17" width="10.5" style="16" customWidth="1"/>
-    <col min="18" max="18" width="42.5" style="16" customWidth="1"/>
+    <col min="17" max="17" width="10.5" style="15" customWidth="1"/>
+    <col min="18" max="18" width="42.5" style="15" customWidth="1"/>
     <col min="19" max="19" width="15.83203125" style="10" customWidth="1"/>
     <col min="20" max="20" width="44.1640625" style="10" customWidth="1"/>
-    <col min="21" max="21" width="44.1640625" style="16" customWidth="1"/>
+    <col min="21" max="21" width="44.1640625" style="15" customWidth="1"/>
     <col min="22" max="23" width="10.83203125" style="6"/>
     <col min="24" max="24" width="14.83203125" style="6" customWidth="1"/>
     <col min="25" max="16384" width="10.83203125" style="6"/>
@@ -3724,19 +3723,19 @@
       <c r="G1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="17" t="s">
+      <c r="H1" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="32" t="s">
+      <c r="I1" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="J1" s="32" t="s">
+      <c r="J1" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="K1" s="32" t="s">
+      <c r="K1" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="L1" s="32" t="s">
+      <c r="L1" s="31" t="s">
         <v>17</v>
       </c>
       <c r="M1" s="3" t="s">
@@ -3751,19 +3750,19 @@
       <c r="P1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="Q1" s="17" t="s">
+      <c r="Q1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="R1" s="17" t="s">
+      <c r="R1" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="S1" s="17" t="s">
+      <c r="S1" s="16" t="s">
         <v>431</v>
       </c>
       <c r="T1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="U1" s="17" t="s">
+      <c r="U1" s="16" t="s">
         <v>25</v>
       </c>
       <c r="Y1" s="6"/>
@@ -3791,11 +3790,11 @@
         <v>428</v>
       </c>
       <c r="R2" s="10"/>
-      <c r="Y2" s="13"/>
+      <c r="Y2" s="12"/>
       <c r="Z2" s="5"/>
       <c r="AA2" s="5"/>
       <c r="AB2" s="5"/>
-      <c r="AC2" s="13"/>
+      <c r="AC2" s="12"/>
       <c r="AD2" s="5"/>
       <c r="AE2" s="5"/>
       <c r="AG2" s="5"/>
@@ -3825,11 +3824,11 @@
         <v>428</v>
       </c>
       <c r="R3" s="10"/>
-      <c r="Y3" s="13"/>
+      <c r="Y3" s="12"/>
       <c r="Z3" s="5"/>
       <c r="AA3" s="5"/>
       <c r="AB3" s="5"/>
-      <c r="AC3" s="13"/>
+      <c r="AC3" s="12"/>
       <c r="AD3" s="5"/>
       <c r="AE3" s="5"/>
     </row>
@@ -3856,11 +3855,11 @@
         <v>428</v>
       </c>
       <c r="R4" s="10"/>
-      <c r="Y4" s="13"/>
+      <c r="Y4" s="12"/>
       <c r="Z4" s="5"/>
       <c r="AA4" s="5"/>
       <c r="AB4" s="5"/>
-      <c r="AC4" s="13"/>
+      <c r="AC4" s="12"/>
       <c r="AD4" s="5"/>
       <c r="AE4" s="5"/>
     </row>
@@ -3886,14 +3885,14 @@
       <c r="P5" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R5" s="16" t="s">
+      <c r="R5" s="15" t="s">
         <v>432</v>
       </c>
-      <c r="Y5" s="13"/>
+      <c r="Y5" s="12"/>
       <c r="Z5" s="5"/>
       <c r="AA5" s="5"/>
       <c r="AB5" s="5"/>
-      <c r="AC5" s="13"/>
+      <c r="AC5" s="12"/>
       <c r="AD5" s="5"/>
       <c r="AE5" s="5"/>
     </row>
@@ -3920,11 +3919,11 @@
         <v>428</v>
       </c>
       <c r="R6" s="10"/>
-      <c r="Y6" s="13"/>
+      <c r="Y6" s="12"/>
       <c r="Z6" s="5"/>
       <c r="AA6" s="5"/>
       <c r="AB6" s="5"/>
-      <c r="AC6" s="13"/>
+      <c r="AC6" s="12"/>
       <c r="AD6" s="5"/>
       <c r="AE6" s="5"/>
     </row>
@@ -3950,15 +3949,15 @@
       <c r="P7" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R7" s="16" t="s">
+      <c r="R7" s="15" t="s">
         <v>432</v>
       </c>
-      <c r="X7" s="14"/>
-      <c r="Y7" s="13"/>
+      <c r="X7" s="13"/>
+      <c r="Y7" s="12"/>
       <c r="Z7" s="5"/>
       <c r="AA7" s="5"/>
       <c r="AB7" s="5"/>
-      <c r="AC7" s="13"/>
+      <c r="AC7" s="12"/>
       <c r="AD7" s="5"/>
       <c r="AE7" s="5"/>
     </row>
@@ -3984,7 +3983,7 @@
       <c r="P8" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R8" s="16" t="s">
+      <c r="R8" s="15" t="s">
         <v>432</v>
       </c>
     </row>
@@ -4133,11 +4132,11 @@
       <c r="G15" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R15" s="16" t="s">
+      <c r="R15" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="16" spans="1:35" ht="51" x14ac:dyDescent="0.2">
@@ -4159,11 +4158,11 @@
       <c r="G16" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R16" s="16" t="s">
+      <c r="R16" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S16" s="10" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="17" spans="1:19" ht="51" x14ac:dyDescent="0.2">
@@ -4289,11 +4288,11 @@
       <c r="G22" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R22" s="16" t="s">
-        <v>438</v>
+      <c r="R22" s="15" t="s">
+        <v>437</v>
       </c>
       <c r="S22" s="10" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="23" spans="1:19" ht="102" x14ac:dyDescent="0.2">
@@ -4315,7 +4314,7 @@
       <c r="G23" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R23" s="16" t="s">
+      <c r="R23" s="15" t="s">
         <v>435</v>
       </c>
       <c r="S23" s="10" t="s">
@@ -4341,7 +4340,7 @@
       <c r="G24" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R24" s="16" t="s">
+      <c r="R24" s="15" t="s">
         <v>434</v>
       </c>
     </row>
@@ -4415,11 +4414,11 @@
       <c r="P27" s="10" t="s">
         <v>430</v>
       </c>
-      <c r="R27" s="16" t="s">
+      <c r="R27" s="15" t="s">
         <v>436</v>
       </c>
       <c r="S27" s="10" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="28" spans="1:19" ht="85" x14ac:dyDescent="0.2">
@@ -4492,11 +4491,11 @@
       <c r="P30" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R30" s="16" t="s">
+      <c r="R30" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S30" s="10" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
     </row>
     <row r="31" spans="1:19" ht="34" x14ac:dyDescent="0.2">
@@ -4521,11 +4520,11 @@
       <c r="P31" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R31" s="16" t="s">
+      <c r="R31" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S31" s="10" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
     </row>
     <row r="32" spans="1:19" ht="34" x14ac:dyDescent="0.2">
@@ -4547,11 +4546,11 @@
       <c r="G32" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R32" s="16" t="s">
+      <c r="R32" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S32" s="10" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
     </row>
     <row r="33" spans="1:19" ht="170" x14ac:dyDescent="0.2">
@@ -4576,11 +4575,11 @@
       <c r="P33" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R33" s="16" t="s">
+      <c r="R33" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S33" s="10" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="34" spans="1:19" ht="119" x14ac:dyDescent="0.2">
@@ -4605,11 +4604,11 @@
       <c r="P34" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R34" s="16" t="s">
+      <c r="R34" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S34" s="10" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="35" spans="1:19" ht="136" x14ac:dyDescent="0.2">
@@ -4634,11 +4633,11 @@
       <c r="P35" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R35" s="16" t="s">
+      <c r="R35" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S35" s="10" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="36" spans="1:19" ht="102" x14ac:dyDescent="0.2">
@@ -4663,11 +4662,11 @@
       <c r="P36" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R36" s="16" t="s">
+      <c r="R36" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S36" s="10" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="37" spans="1:19" ht="85" x14ac:dyDescent="0.2">
@@ -4692,11 +4691,11 @@
       <c r="P37" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R37" s="16" t="s">
+      <c r="R37" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S37" s="10" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="38" spans="1:19" ht="85" x14ac:dyDescent="0.2">
@@ -4721,11 +4720,11 @@
       <c r="P38" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R38" s="16" t="s">
+      <c r="R38" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S38" s="10" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="39" spans="1:19" ht="68" x14ac:dyDescent="0.2">
@@ -4750,11 +4749,11 @@
       <c r="P39" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R39" s="16" t="s">
+      <c r="R39" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S39" s="10" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="40" spans="1:19" ht="85" x14ac:dyDescent="0.2">
@@ -4818,11 +4817,11 @@
       <c r="G42" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="R42" s="16" t="s">
+      <c r="R42" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S42" s="10" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="43" spans="1:19" ht="51" x14ac:dyDescent="0.2">
@@ -4886,11 +4885,11 @@
       <c r="G45" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="R45" s="16" t="s">
-        <v>443</v>
+      <c r="R45" s="15" t="s">
+        <v>436</v>
       </c>
       <c r="S45" s="10" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="46" spans="1:19" ht="68" x14ac:dyDescent="0.2">
@@ -4956,7 +4955,7 @@
       </c>
       <c r="R48" s="10"/>
     </row>
-    <row r="49" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="s">
         <v>167</v>
       </c>
@@ -4975,14 +4974,14 @@
       <c r="G49" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R49" s="16" t="s">
+      <c r="R49" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S49" s="10" t="s">
         <v>444</v>
       </c>
     </row>
-    <row r="50" spans="1:19" ht="102" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:21" ht="102" x14ac:dyDescent="0.2">
       <c r="A50" s="7" t="s">
         <v>169</v>
       </c>
@@ -5003,7 +5002,7 @@
       </c>
       <c r="R50" s="10"/>
     </row>
-    <row r="51" spans="1:19" ht="153" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:21" ht="153" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
         <v>171</v>
       </c>
@@ -5024,7 +5023,7 @@
       </c>
       <c r="R51" s="10"/>
     </row>
-    <row r="52" spans="1:19" ht="17" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:21" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="7" t="s">
         <v>173</v>
       </c>
@@ -5038,16 +5037,22 @@
         <v>26</v>
       </c>
       <c r="E52" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G52" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R52" s="10" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="53" spans="1:19" ht="102" x14ac:dyDescent="0.2">
+      <c r="R52" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="S52" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="U52" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="53" spans="1:21" ht="102" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
         <v>175</v>
       </c>
@@ -5061,16 +5066,22 @@
         <v>26</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G53" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R53" s="10" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="54" spans="1:19" ht="102" x14ac:dyDescent="0.2">
+      <c r="R53" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="S53" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="U53" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="54" spans="1:21" ht="102" x14ac:dyDescent="0.2">
       <c r="A54" s="7" t="s">
         <v>177</v>
       </c>
@@ -5084,16 +5095,22 @@
         <v>26</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G54" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R54" s="10" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="55" spans="1:19" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R54" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="S54" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="U54" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="55" spans="1:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
         <v>179</v>
       </c>
@@ -5107,16 +5124,22 @@
         <v>26</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G55" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R55" s="10" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="56" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+      <c r="R55" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="S55" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="U55" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="56" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
         <v>181</v>
       </c>
@@ -5135,9 +5158,8 @@
       <c r="G56" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R56" s="10"/>
-    </row>
-    <row r="57" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    </row>
+    <row r="57" spans="1:21" ht="85" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
         <v>183</v>
       </c>
@@ -5145,22 +5167,28 @@
         <v>184</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>448</v>
+        <v>438</v>
       </c>
       <c r="D57" s="7" t="s">
         <v>26</v>
       </c>
       <c r="E57" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G57" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R57" s="10" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="58" spans="1:19" ht="102" x14ac:dyDescent="0.2">
+      <c r="R57" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="S57" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="U57" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="58" spans="1:21" ht="102" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="s">
         <v>185</v>
       </c>
@@ -5174,16 +5202,22 @@
         <v>26</v>
       </c>
       <c r="E58" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G58" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R58" s="10" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="59" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+      <c r="R58" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="S58" s="10" t="s">
+        <v>443</v>
+      </c>
+      <c r="U58" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="59" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A59" s="7" t="s">
         <v>187</v>
       </c>
@@ -5197,16 +5231,22 @@
         <v>26</v>
       </c>
       <c r="E59" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G59" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R59" s="10" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="60" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+      <c r="R59" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="S59" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="U59" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="60" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A60" s="7" t="s">
         <v>189</v>
       </c>
@@ -5220,16 +5260,22 @@
         <v>26</v>
       </c>
       <c r="E60" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G60" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R60" s="10" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="61" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+      <c r="R60" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="S60" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="U60" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="61" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A61" s="7" t="s">
         <v>191</v>
       </c>
@@ -5243,16 +5289,22 @@
         <v>26</v>
       </c>
       <c r="E61" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G61" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R61" s="10" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="62" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+      <c r="R61" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="S61" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="U61" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="62" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A62" s="7" t="s">
         <v>193</v>
       </c>
@@ -5271,9 +5323,8 @@
       <c r="G62" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R62" s="10"/>
-    </row>
-    <row r="63" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    </row>
+    <row r="63" spans="1:21" ht="34" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
         <v>195</v>
       </c>
@@ -5287,16 +5338,22 @@
         <v>26</v>
       </c>
       <c r="E63" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G63" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R63" s="10" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="64" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+      <c r="R63" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="S63" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="U63" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="64" spans="1:21" ht="34" x14ac:dyDescent="0.2">
       <c r="A64" s="7" t="s">
         <v>197</v>
       </c>
@@ -5310,16 +5367,22 @@
         <v>26</v>
       </c>
       <c r="E64" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G64" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R64" s="10" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="65" spans="1:19" ht="102" x14ac:dyDescent="0.2">
+      <c r="R64" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="S64" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="U64" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="65" spans="1:21" ht="102" x14ac:dyDescent="0.2">
       <c r="A65" s="7" t="s">
         <v>199</v>
       </c>
@@ -5340,7 +5403,7 @@
       </c>
       <c r="R65" s="10"/>
     </row>
-    <row r="66" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:21" ht="85" x14ac:dyDescent="0.2">
       <c r="A66" s="7" t="s">
         <v>201</v>
       </c>
@@ -5361,7 +5424,7 @@
       </c>
       <c r="R66" s="10"/>
     </row>
-    <row r="67" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="s">
         <v>203</v>
       </c>
@@ -5380,14 +5443,14 @@
       <c r="G67" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R67" s="16" t="s">
+      <c r="R67" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S67" s="10" t="s">
         <v>444</v>
       </c>
     </row>
-    <row r="68" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A68" s="7" t="s">
         <v>205</v>
       </c>
@@ -5408,7 +5471,7 @@
       </c>
       <c r="R68" s="10"/>
     </row>
-    <row r="69" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:21" ht="85" x14ac:dyDescent="0.2">
       <c r="A69" s="7" t="s">
         <v>207</v>
       </c>
@@ -5429,7 +5492,7 @@
       </c>
       <c r="R69" s="10"/>
     </row>
-    <row r="70" spans="1:19" ht="119" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:21" ht="119" x14ac:dyDescent="0.2">
       <c r="A70" s="7" t="s">
         <v>209</v>
       </c>
@@ -5450,7 +5513,7 @@
       </c>
       <c r="R70" s="10"/>
     </row>
-    <row r="71" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A71" s="7" t="s">
         <v>211</v>
       </c>
@@ -5471,7 +5534,7 @@
       </c>
       <c r="R71" s="10"/>
     </row>
-    <row r="72" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:21" ht="34" x14ac:dyDescent="0.2">
       <c r="A72" s="7" t="s">
         <v>213</v>
       </c>
@@ -5492,7 +5555,7 @@
       </c>
       <c r="R72" s="10"/>
     </row>
-    <row r="73" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A73" s="7" t="s">
         <v>215</v>
       </c>
@@ -5513,7 +5576,7 @@
       </c>
       <c r="R73" s="10"/>
     </row>
-    <row r="74" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:21" ht="85" x14ac:dyDescent="0.2">
       <c r="A74" s="7" t="s">
         <v>217</v>
       </c>
@@ -5534,7 +5597,7 @@
       </c>
       <c r="R74" s="10"/>
     </row>
-    <row r="75" spans="1:19" ht="102" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:21" ht="102" x14ac:dyDescent="0.2">
       <c r="A75" s="7" t="s">
         <v>219</v>
       </c>
@@ -5555,7 +5618,7 @@
       </c>
       <c r="R75" s="10"/>
     </row>
-    <row r="76" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="s">
         <v>221</v>
       </c>
@@ -5569,16 +5632,16 @@
         <v>26</v>
       </c>
       <c r="E76" s="7" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="G76" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R76" s="16" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="77" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+      <c r="U76" s="15" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="77" spans="1:21" ht="85" x14ac:dyDescent="0.2">
       <c r="A77" s="7" t="s">
         <v>223</v>
       </c>
@@ -5599,7 +5662,7 @@
       </c>
       <c r="R77" s="10"/>
     </row>
-    <row r="78" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:21" ht="34" x14ac:dyDescent="0.2">
       <c r="A78" s="7" t="s">
         <v>225</v>
       </c>
@@ -5620,7 +5683,7 @@
       </c>
       <c r="R78" s="10"/>
     </row>
-    <row r="79" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A79" s="7" t="s">
         <v>227</v>
       </c>
@@ -5641,7 +5704,7 @@
       </c>
       <c r="R79" s="10"/>
     </row>
-    <row r="80" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A80" s="7" t="s">
         <v>229</v>
       </c>
@@ -5662,7 +5725,7 @@
       </c>
       <c r="R80" s="10"/>
     </row>
-    <row r="81" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A81" s="7" t="s">
         <v>231</v>
       </c>
@@ -5683,7 +5746,7 @@
       </c>
       <c r="R81" s="10"/>
     </row>
-    <row r="82" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A82" s="7" t="s">
         <v>233</v>
       </c>
@@ -5704,7 +5767,7 @@
       </c>
       <c r="R82" s="10"/>
     </row>
-    <row r="83" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A83" s="7" t="s">
         <v>235</v>
       </c>
@@ -5725,7 +5788,7 @@
       </c>
       <c r="R83" s="10"/>
     </row>
-    <row r="84" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:21" ht="34" x14ac:dyDescent="0.2">
       <c r="A84" s="7" t="s">
         <v>237</v>
       </c>
@@ -5746,7 +5809,7 @@
       </c>
       <c r="R84" s="10"/>
     </row>
-    <row r="85" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="s">
         <v>239</v>
       </c>
@@ -5767,7 +5830,7 @@
       </c>
       <c r="R85" s="10"/>
     </row>
-    <row r="86" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A86" s="7" t="s">
         <v>241</v>
       </c>
@@ -5788,7 +5851,7 @@
       </c>
       <c r="R86" s="10"/>
     </row>
-    <row r="87" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A87" s="7" t="s">
         <v>243</v>
       </c>
@@ -5809,7 +5872,7 @@
       </c>
       <c r="R87" s="10"/>
     </row>
-    <row r="88" spans="1:19" ht="136" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:21" ht="136" x14ac:dyDescent="0.2">
       <c r="A88" s="7" t="s">
         <v>245</v>
       </c>
@@ -5823,19 +5886,16 @@
         <v>26</v>
       </c>
       <c r="E88" s="7" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="G88" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R88" s="16" t="s">
-        <v>446</v>
-      </c>
-      <c r="S88" s="10" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="89" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+      <c r="U88" s="15" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="89" spans="1:21" ht="85" x14ac:dyDescent="0.2">
       <c r="A89" s="7" t="s">
         <v>247</v>
       </c>
@@ -5856,7 +5916,7 @@
       </c>
       <c r="R89" s="10"/>
     </row>
-    <row r="90" spans="1:19" ht="136" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:21" ht="136" x14ac:dyDescent="0.2">
       <c r="A90" s="7" t="s">
         <v>249</v>
       </c>
@@ -5877,7 +5937,7 @@
       </c>
       <c r="R90" s="10"/>
     </row>
-    <row r="91" spans="1:19" ht="102" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:21" ht="102" x14ac:dyDescent="0.2">
       <c r="A91" s="7" t="s">
         <v>251</v>
       </c>
@@ -5898,7 +5958,7 @@
       </c>
       <c r="R91" s="10"/>
     </row>
-    <row r="92" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:21" ht="34" x14ac:dyDescent="0.2">
       <c r="A92" s="7" t="s">
         <v>253</v>
       </c>
@@ -5919,7 +5979,7 @@
       </c>
       <c r="R92" s="10"/>
     </row>
-    <row r="93" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A93" s="7" t="s">
         <v>255</v>
       </c>
@@ -5940,7 +6000,7 @@
       </c>
       <c r="R93" s="10"/>
     </row>
-    <row r="94" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:21" ht="85" x14ac:dyDescent="0.2">
       <c r="A94" s="7" t="s">
         <v>257</v>
       </c>
@@ -5961,7 +6021,7 @@
       </c>
       <c r="R94" s="10"/>
     </row>
-    <row r="95" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:21" ht="85" x14ac:dyDescent="0.2">
       <c r="A95" s="7" t="s">
         <v>259</v>
       </c>
@@ -5982,7 +6042,7 @@
       </c>
       <c r="R95" s="10"/>
     </row>
-    <row r="96" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:21" ht="34" x14ac:dyDescent="0.2">
       <c r="A96" s="7" t="s">
         <v>261</v>
       </c>
@@ -5998,13 +6058,13 @@
       <c r="E96" s="7" t="s">
         <v>424</v>
       </c>
-      <c r="F96" s="29"/>
+      <c r="F96" s="28"/>
       <c r="G96" s="7" t="b">
         <v>0</v>
       </c>
       <c r="R96" s="10"/>
     </row>
-    <row r="97" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A97" s="7" t="s">
         <v>263</v>
       </c>
@@ -6025,7 +6085,7 @@
       </c>
       <c r="R97" s="10"/>
     </row>
-    <row r="98" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A98" s="7" t="s">
         <v>265</v>
       </c>
@@ -6039,16 +6099,22 @@
         <v>26</v>
       </c>
       <c r="E98" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G98" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R98" s="10" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="99" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+      <c r="R98" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="S98" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="U98" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="99" spans="1:21" ht="34" x14ac:dyDescent="0.2">
       <c r="A99" s="7" t="s">
         <v>267</v>
       </c>
@@ -6061,17 +6127,23 @@
       <c r="D99" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E99" s="12" t="s">
-        <v>424</v>
+      <c r="E99" s="7" t="s">
+        <v>425</v>
       </c>
       <c r="G99" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R99" s="10" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="100" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+      <c r="R99" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="S99" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="U99" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="100" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A100" s="7" t="s">
         <v>269</v>
       </c>
@@ -6092,7 +6164,7 @@
       </c>
       <c r="R100" s="10"/>
     </row>
-    <row r="101" spans="1:19" ht="136" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:21" ht="136" x14ac:dyDescent="0.2">
       <c r="A101" s="7" t="s">
         <v>271</v>
       </c>
@@ -6113,7 +6185,7 @@
       </c>
       <c r="R101" s="10"/>
     </row>
-    <row r="102" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:21" ht="34" x14ac:dyDescent="0.2">
       <c r="A102" s="7" t="s">
         <v>273</v>
       </c>
@@ -6134,7 +6206,7 @@
       </c>
       <c r="R102" s="10"/>
     </row>
-    <row r="103" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:21" ht="85" x14ac:dyDescent="0.2">
       <c r="A103" s="7" t="s">
         <v>275</v>
       </c>
@@ -6153,14 +6225,14 @@
       <c r="G103" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R103" s="16" t="s">
+      <c r="R103" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S103" s="10" t="s">
         <v>444</v>
       </c>
     </row>
-    <row r="104" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:21" ht="85" x14ac:dyDescent="0.2">
       <c r="A104" s="7" t="s">
         <v>277</v>
       </c>
@@ -6181,7 +6253,7 @@
       </c>
       <c r="R104" s="10"/>
     </row>
-    <row r="105" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A105" s="7" t="s">
         <v>279</v>
       </c>
@@ -6202,7 +6274,7 @@
       </c>
       <c r="R105" s="10"/>
     </row>
-    <row r="106" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A106" s="7" t="s">
         <v>281</v>
       </c>
@@ -6216,16 +6288,22 @@
         <v>26</v>
       </c>
       <c r="E106" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G106" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R106" s="10" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="107" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+      <c r="R106" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="S106" s="10" t="s">
+        <v>442</v>
+      </c>
+      <c r="U106" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="107" spans="1:21" ht="34" x14ac:dyDescent="0.2">
       <c r="A107" s="7" t="s">
         <v>283</v>
       </c>
@@ -6239,16 +6317,22 @@
         <v>35</v>
       </c>
       <c r="E107" s="7" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G107" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R107" s="10" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="108" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+      <c r="R107" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="S107" s="10" t="s">
+        <v>442</v>
+      </c>
+      <c r="U107" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="108" spans="1:21" ht="34" x14ac:dyDescent="0.2">
       <c r="A108" s="7" t="s">
         <v>285</v>
       </c>
@@ -6261,17 +6345,23 @@
       <c r="D108" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E108" s="42" t="s">
-        <v>424</v>
+      <c r="E108" s="7" t="s">
+        <v>425</v>
       </c>
       <c r="G108" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R108" s="10" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="109" spans="1:19" ht="102" x14ac:dyDescent="0.2">
+      <c r="R108" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="S108" s="10" t="s">
+        <v>442</v>
+      </c>
+      <c r="U108" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="109" spans="1:21" ht="102" x14ac:dyDescent="0.2">
       <c r="A109" s="7" t="s">
         <v>287</v>
       </c>
@@ -6290,14 +6380,14 @@
       <c r="G109" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R109" s="16" t="s">
+      <c r="R109" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S109" s="10" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="110" spans="1:19" ht="119" x14ac:dyDescent="0.2">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="110" spans="1:21" ht="119" x14ac:dyDescent="0.2">
       <c r="A110" s="7" t="s">
         <v>289</v>
       </c>
@@ -6310,20 +6400,20 @@
       <c r="D110" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E110" s="42" t="s">
+      <c r="E110" s="41" t="s">
         <v>426</v>
       </c>
       <c r="G110" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R110" s="16" t="s">
+      <c r="R110" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S110" s="10" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="111" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="111" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A111" s="7" t="s">
         <v>291</v>
       </c>
@@ -6336,20 +6426,20 @@
       <c r="D111" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E111" s="42" t="s">
+      <c r="E111" s="41" t="s">
         <v>426</v>
       </c>
       <c r="G111" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R111" s="16" t="s">
+      <c r="R111" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S111" s="10" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="112" spans="1:19" ht="119" x14ac:dyDescent="0.2">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="112" spans="1:21" ht="119" x14ac:dyDescent="0.2">
       <c r="A112" s="7" t="s">
         <v>293</v>
       </c>
@@ -6362,20 +6452,20 @@
       <c r="D112" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E112" s="42" t="s">
+      <c r="E112" s="41" t="s">
         <v>426</v>
       </c>
       <c r="G112" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R112" s="16" t="s">
+      <c r="R112" s="15" t="s">
         <v>433</v>
       </c>
       <c r="S112" s="10" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="113" spans="1:19" ht="102" x14ac:dyDescent="0.2">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="113" spans="1:21" ht="102" x14ac:dyDescent="0.2">
       <c r="A113" s="7" t="s">
         <v>295</v>
       </c>
@@ -6388,17 +6478,23 @@
       <c r="D113" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E113" s="42" t="s">
-        <v>424</v>
+      <c r="E113" s="7" t="s">
+        <v>425</v>
       </c>
       <c r="G113" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R113" s="10" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="114" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+      <c r="R113" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="S113" s="10" t="s">
+        <v>442</v>
+      </c>
+      <c r="U113" s="15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="114" spans="1:21" ht="85" x14ac:dyDescent="0.2">
       <c r="A114" s="7" t="s">
         <v>297</v>
       </c>
@@ -6411,7 +6507,7 @@
       <c r="D114" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E114" s="42" t="s">
+      <c r="E114" s="41" t="s">
         <v>424</v>
       </c>
       <c r="G114" s="7" t="b">
@@ -6419,7 +6515,7 @@
       </c>
       <c r="R114" s="10"/>
     </row>
-    <row r="115" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:21" ht="34" x14ac:dyDescent="0.2">
       <c r="A115" s="7" t="s">
         <v>299</v>
       </c>
@@ -6432,7 +6528,7 @@
       <c r="D115" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E115" s="42" t="s">
+      <c r="E115" s="41" t="s">
         <v>424</v>
       </c>
       <c r="G115" s="7" t="b">
@@ -6443,7 +6539,7 @@
       </c>
       <c r="R115" s="10"/>
     </row>
-    <row r="116" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A116" s="7" t="s">
         <v>301</v>
       </c>
@@ -6456,7 +6552,7 @@
       <c r="D116" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E116" s="42" t="s">
+      <c r="E116" s="41" t="s">
         <v>424</v>
       </c>
       <c r="G116" s="7" t="b">
@@ -6467,7 +6563,7 @@
       </c>
       <c r="R116" s="10"/>
     </row>
-    <row r="117" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:21" ht="85" x14ac:dyDescent="0.2">
       <c r="A117" s="7" t="s">
         <v>303</v>
       </c>
@@ -6491,7 +6587,7 @@
       </c>
       <c r="R117" s="10"/>
     </row>
-    <row r="118" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A118" s="7" t="s">
         <v>305</v>
       </c>
@@ -6515,7 +6611,7 @@
       </c>
       <c r="R118" s="10"/>
     </row>
-    <row r="119" spans="1:19" ht="170" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:21" ht="170" x14ac:dyDescent="0.2">
       <c r="A119" s="7" t="s">
         <v>307</v>
       </c>
@@ -6537,14 +6633,14 @@
       <c r="P119" s="10" t="s">
         <v>430</v>
       </c>
-      <c r="R119" s="16" t="s">
+      <c r="R119" s="15" t="s">
         <v>436</v>
       </c>
       <c r="S119" s="10" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="120" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="120" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A120" s="7" t="s">
         <v>309</v>
       </c>
@@ -6568,82 +6664,82 @@
       </c>
       <c r="R120" s="10"/>
     </row>
-    <row r="121" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B121" s="11"/>
       <c r="R121" s="10"/>
     </row>
-    <row r="122" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B122" s="11"/>
       <c r="R122" s="10"/>
     </row>
-    <row r="123" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B123" s="11"/>
-      <c r="I123" s="31"/>
-      <c r="J123" s="31"/>
-      <c r="K123" s="31"/>
-      <c r="L123" s="31"/>
+      <c r="I123" s="30"/>
+      <c r="J123" s="30"/>
+      <c r="K123" s="30"/>
+      <c r="L123" s="30"/>
       <c r="Q123" s="10"/>
       <c r="R123" s="10"/>
     </row>
-    <row r="124" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B124" s="11"/>
-      <c r="E124" s="42"/>
+      <c r="E124" s="41"/>
       <c r="R124" s="10"/>
     </row>
-    <row r="125" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B125" s="11"/>
       <c r="R125" s="10"/>
     </row>
-    <row r="126" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B126" s="11"/>
       <c r="R126" s="10"/>
     </row>
-    <row r="127" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B127" s="11"/>
       <c r="R127" s="10"/>
     </row>
-    <row r="128" spans="1:19" ht="16" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B128" s="11"/>
       <c r="R128" s="10"/>
     </row>
     <row r="129" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B129" s="11"/>
-      <c r="E129" s="42"/>
+      <c r="E129" s="41"/>
       <c r="R129" s="10"/>
     </row>
     <row r="130" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B130" s="11"/>
-      <c r="E130" s="42"/>
+      <c r="E130" s="41"/>
       <c r="R130" s="10"/>
     </row>
     <row r="131" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B131" s="11"/>
-      <c r="E131" s="42"/>
+      <c r="E131" s="41"/>
       <c r="R131" s="10"/>
     </row>
     <row r="132" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B132" s="11"/>
-      <c r="E132" s="42"/>
+      <c r="E132" s="41"/>
       <c r="R132" s="10"/>
     </row>
     <row r="133" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B133" s="11"/>
-      <c r="E133" s="42"/>
+      <c r="E133" s="41"/>
       <c r="R133" s="10"/>
     </row>
     <row r="134" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B134" s="11"/>
-      <c r="E134" s="42"/>
+      <c r="E134" s="41"/>
       <c r="R134" s="10"/>
     </row>
     <row r="135" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B135" s="11"/>
-      <c r="E135" s="42"/>
+      <c r="E135" s="41"/>
       <c r="R135" s="10"/>
     </row>
     <row r="136" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B136" s="11"/>
-      <c r="E136" s="42"/>
+      <c r="E136" s="41"/>
       <c r="R136" s="10"/>
     </row>
     <row r="137" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6652,12 +6748,12 @@
     </row>
     <row r="138" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B138" s="11"/>
-      <c r="E138" s="42"/>
+      <c r="E138" s="41"/>
       <c r="R138" s="10"/>
     </row>
     <row r="139" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B139" s="11"/>
-      <c r="E139" s="42"/>
+      <c r="E139" s="41"/>
       <c r="R139" s="10"/>
     </row>
     <row r="140" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6666,7 +6762,7 @@
     </row>
     <row r="141" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B141" s="11"/>
-      <c r="E141" s="42"/>
+      <c r="E141" s="41"/>
       <c r="R141" s="10"/>
     </row>
     <row r="142" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6683,7 +6779,7 @@
     </row>
     <row r="145" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B145" s="11"/>
-      <c r="E145" s="42"/>
+      <c r="E145" s="41"/>
       <c r="R145" s="10"/>
     </row>
     <row r="146" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6692,32 +6788,32 @@
     </row>
     <row r="147" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B147" s="11"/>
-      <c r="E147" s="42"/>
+      <c r="E147" s="41"/>
       <c r="R147" s="10"/>
     </row>
     <row r="148" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B148" s="11"/>
-      <c r="E148" s="42"/>
+      <c r="E148" s="41"/>
       <c r="R148" s="10"/>
     </row>
     <row r="149" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B149" s="11"/>
-      <c r="E149" s="42"/>
+      <c r="E149" s="41"/>
       <c r="R149" s="10"/>
     </row>
     <row r="150" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B150" s="11"/>
-      <c r="E150" s="42"/>
+      <c r="E150" s="41"/>
       <c r="R150" s="10"/>
     </row>
     <row r="151" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B151" s="11"/>
-      <c r="E151" s="42"/>
+      <c r="E151" s="41"/>
       <c r="R151" s="10"/>
     </row>
     <row r="152" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B152" s="11"/>
-      <c r="E152" s="42"/>
+      <c r="E152" s="41"/>
       <c r="R152" s="10"/>
     </row>
     <row r="153" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6814,42 +6910,42 @@
     </row>
     <row r="176" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B176" s="11"/>
-      <c r="E176" s="42"/>
+      <c r="E176" s="41"/>
       <c r="R176" s="10"/>
     </row>
     <row r="177" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B177" s="11"/>
-      <c r="E177" s="42"/>
+      <c r="E177" s="41"/>
       <c r="R177" s="10"/>
     </row>
     <row r="178" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B178" s="11"/>
-      <c r="E178" s="42"/>
+      <c r="E178" s="41"/>
       <c r="R178" s="10"/>
     </row>
     <row r="179" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B179" s="11"/>
-      <c r="E179" s="42"/>
+      <c r="E179" s="41"/>
       <c r="R179" s="10"/>
     </row>
     <row r="180" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B180" s="11"/>
-      <c r="E180" s="42"/>
+      <c r="E180" s="41"/>
       <c r="R180" s="10"/>
     </row>
     <row r="181" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B181" s="11"/>
-      <c r="E181" s="42"/>
+      <c r="E181" s="41"/>
       <c r="R181" s="10"/>
     </row>
     <row r="182" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B182" s="11"/>
-      <c r="E182" s="42"/>
+      <c r="E182" s="41"/>
       <c r="R182" s="10"/>
     </row>
     <row r="183" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B183" s="11"/>
-      <c r="E183" s="42"/>
+      <c r="E183" s="41"/>
       <c r="R183" s="10"/>
     </row>
     <row r="184" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6858,7 +6954,7 @@
     </row>
     <row r="185" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B185" s="11"/>
-      <c r="E185" s="42"/>
+      <c r="E185" s="41"/>
       <c r="R185" s="10"/>
     </row>
     <row r="186" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6875,7 +6971,7 @@
     </row>
     <row r="189" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B189" s="11"/>
-      <c r="E189" s="42"/>
+      <c r="E189" s="41"/>
       <c r="R189" s="10"/>
     </row>
     <row r="190" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6888,12 +6984,12 @@
     </row>
     <row r="192" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B192" s="11"/>
-      <c r="E192" s="42"/>
+      <c r="E192" s="41"/>
       <c r="R192" s="10"/>
     </row>
     <row r="193" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B193" s="11"/>
-      <c r="E193" s="42"/>
+      <c r="E193" s="41"/>
       <c r="R193" s="10"/>
     </row>
     <row r="194" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6914,7 +7010,7 @@
     </row>
     <row r="198" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B198" s="11"/>
-      <c r="E198" s="42"/>
+      <c r="E198" s="41"/>
       <c r="R198" s="10"/>
     </row>
     <row r="199" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6955,25 +7051,25 @@
     </row>
     <row r="208" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B208" s="11"/>
-      <c r="E208" s="42"/>
+      <c r="E208" s="41"/>
       <c r="R208" s="10"/>
     </row>
     <row r="209" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B209" s="11"/>
-      <c r="E209" s="42"/>
+      <c r="E209" s="41"/>
       <c r="R209" s="10"/>
     </row>
     <row r="210" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B210" s="11"/>
-      <c r="E210" s="42"/>
+      <c r="E210" s="41"/>
       <c r="R210" s="10"/>
     </row>
     <row r="211" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B211" s="11"/>
-      <c r="E211" s="42"/>
+      <c r="E211" s="41"/>
       <c r="R211" s="10"/>
     </row>
-    <row r="212" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A212" s="7"/>
       <c r="B212" s="11"/>
       <c r="C212" s="8"/>
@@ -6981,22 +7077,22 @@
       <c r="E212" s="8"/>
       <c r="F212" s="8"/>
       <c r="G212" s="8"/>
-      <c r="H212" s="16"/>
-      <c r="I212" s="30"/>
-      <c r="J212" s="30"/>
-      <c r="K212" s="30"/>
-      <c r="L212" s="30"/>
-      <c r="M212" s="43"/>
-      <c r="N212" s="43"/>
-      <c r="O212" s="16"/>
-      <c r="P212" s="16"/>
-      <c r="Q212" s="16"/>
-      <c r="R212" s="16"/>
-      <c r="S212" s="16"/>
-      <c r="T212" s="16"/>
-      <c r="U212" s="16"/>
-    </row>
-    <row r="213" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H212" s="15"/>
+      <c r="I212" s="29"/>
+      <c r="J212" s="29"/>
+      <c r="K212" s="29"/>
+      <c r="L212" s="29"/>
+      <c r="M212" s="42"/>
+      <c r="N212" s="42"/>
+      <c r="O212" s="15"/>
+      <c r="P212" s="15"/>
+      <c r="Q212" s="15"/>
+      <c r="R212" s="15"/>
+      <c r="S212" s="15"/>
+      <c r="T212" s="15"/>
+      <c r="U212" s="15"/>
+    </row>
+    <row r="213" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A213" s="7"/>
       <c r="B213" s="11"/>
       <c r="C213" s="8"/>
@@ -7004,22 +7100,22 @@
       <c r="E213" s="8"/>
       <c r="F213" s="8"/>
       <c r="G213" s="8"/>
-      <c r="H213" s="16"/>
-      <c r="I213" s="30"/>
-      <c r="J213" s="30"/>
-      <c r="K213" s="30"/>
-      <c r="L213" s="30"/>
-      <c r="M213" s="43"/>
-      <c r="N213" s="43"/>
-      <c r="O213" s="16"/>
-      <c r="P213" s="16"/>
-      <c r="Q213" s="16"/>
-      <c r="R213" s="16"/>
-      <c r="S213" s="16"/>
-      <c r="T213" s="16"/>
-      <c r="U213" s="16"/>
-    </row>
-    <row r="214" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H213" s="15"/>
+      <c r="I213" s="29"/>
+      <c r="J213" s="29"/>
+      <c r="K213" s="29"/>
+      <c r="L213" s="29"/>
+      <c r="M213" s="42"/>
+      <c r="N213" s="42"/>
+      <c r="O213" s="15"/>
+      <c r="P213" s="15"/>
+      <c r="Q213" s="15"/>
+      <c r="R213" s="15"/>
+      <c r="S213" s="15"/>
+      <c r="T213" s="15"/>
+      <c r="U213" s="15"/>
+    </row>
+    <row r="214" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A214" s="7"/>
       <c r="B214" s="11"/>
       <c r="C214" s="8"/>
@@ -7027,22 +7123,22 @@
       <c r="E214" s="8"/>
       <c r="F214" s="8"/>
       <c r="G214" s="8"/>
-      <c r="H214" s="16"/>
-      <c r="I214" s="30"/>
-      <c r="J214" s="30"/>
-      <c r="K214" s="30"/>
-      <c r="L214" s="30"/>
-      <c r="M214" s="43"/>
-      <c r="N214" s="43"/>
-      <c r="O214" s="16"/>
-      <c r="P214" s="16"/>
-      <c r="Q214" s="16"/>
-      <c r="R214" s="16"/>
-      <c r="S214" s="16"/>
-      <c r="T214" s="16"/>
-      <c r="U214" s="16"/>
-    </row>
-    <row r="215" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H214" s="15"/>
+      <c r="I214" s="29"/>
+      <c r="J214" s="29"/>
+      <c r="K214" s="29"/>
+      <c r="L214" s="29"/>
+      <c r="M214" s="42"/>
+      <c r="N214" s="42"/>
+      <c r="O214" s="15"/>
+      <c r="P214" s="15"/>
+      <c r="Q214" s="15"/>
+      <c r="R214" s="15"/>
+      <c r="S214" s="15"/>
+      <c r="T214" s="15"/>
+      <c r="U214" s="15"/>
+    </row>
+    <row r="215" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A215" s="7"/>
       <c r="B215" s="11"/>
       <c r="C215" s="8"/>
@@ -7050,22 +7146,22 @@
       <c r="E215" s="8"/>
       <c r="F215" s="8"/>
       <c r="G215" s="8"/>
-      <c r="H215" s="16"/>
-      <c r="I215" s="30"/>
-      <c r="J215" s="30"/>
-      <c r="K215" s="30"/>
-      <c r="L215" s="30"/>
-      <c r="M215" s="43"/>
-      <c r="N215" s="43"/>
-      <c r="O215" s="16"/>
-      <c r="P215" s="16"/>
-      <c r="Q215" s="16"/>
-      <c r="R215" s="16"/>
-      <c r="S215" s="16"/>
-      <c r="T215" s="16"/>
-      <c r="U215" s="16"/>
-    </row>
-    <row r="216" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H215" s="15"/>
+      <c r="I215" s="29"/>
+      <c r="J215" s="29"/>
+      <c r="K215" s="29"/>
+      <c r="L215" s="29"/>
+      <c r="M215" s="42"/>
+      <c r="N215" s="42"/>
+      <c r="O215" s="15"/>
+      <c r="P215" s="15"/>
+      <c r="Q215" s="15"/>
+      <c r="R215" s="15"/>
+      <c r="S215" s="15"/>
+      <c r="T215" s="15"/>
+      <c r="U215" s="15"/>
+    </row>
+    <row r="216" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A216" s="7"/>
       <c r="B216" s="11"/>
       <c r="C216" s="8"/>
@@ -7073,22 +7169,22 @@
       <c r="E216" s="8"/>
       <c r="F216" s="8"/>
       <c r="G216" s="8"/>
-      <c r="H216" s="16"/>
-      <c r="I216" s="30"/>
-      <c r="J216" s="30"/>
-      <c r="K216" s="30"/>
-      <c r="L216" s="30"/>
-      <c r="M216" s="43"/>
-      <c r="N216" s="43"/>
-      <c r="O216" s="16"/>
-      <c r="P216" s="16"/>
-      <c r="Q216" s="16"/>
-      <c r="R216" s="16"/>
-      <c r="S216" s="16"/>
-      <c r="T216" s="16"/>
-      <c r="U216" s="16"/>
-    </row>
-    <row r="217" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H216" s="15"/>
+      <c r="I216" s="29"/>
+      <c r="J216" s="29"/>
+      <c r="K216" s="29"/>
+      <c r="L216" s="29"/>
+      <c r="M216" s="42"/>
+      <c r="N216" s="42"/>
+      <c r="O216" s="15"/>
+      <c r="P216" s="15"/>
+      <c r="Q216" s="15"/>
+      <c r="R216" s="15"/>
+      <c r="S216" s="15"/>
+      <c r="T216" s="15"/>
+      <c r="U216" s="15"/>
+    </row>
+    <row r="217" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A217" s="7"/>
       <c r="B217" s="11"/>
       <c r="C217" s="8"/>
@@ -7096,22 +7192,22 @@
       <c r="E217" s="8"/>
       <c r="F217" s="8"/>
       <c r="G217" s="8"/>
-      <c r="H217" s="16"/>
-      <c r="I217" s="30"/>
-      <c r="J217" s="30"/>
-      <c r="K217" s="30"/>
-      <c r="L217" s="30"/>
-      <c r="M217" s="43"/>
-      <c r="N217" s="43"/>
-      <c r="O217" s="16"/>
-      <c r="P217" s="16"/>
-      <c r="Q217" s="16"/>
-      <c r="R217" s="16"/>
-      <c r="S217" s="16"/>
-      <c r="T217" s="16"/>
-      <c r="U217" s="16"/>
-    </row>
-    <row r="218" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H217" s="15"/>
+      <c r="I217" s="29"/>
+      <c r="J217" s="29"/>
+      <c r="K217" s="29"/>
+      <c r="L217" s="29"/>
+      <c r="M217" s="42"/>
+      <c r="N217" s="42"/>
+      <c r="O217" s="15"/>
+      <c r="P217" s="15"/>
+      <c r="Q217" s="15"/>
+      <c r="R217" s="15"/>
+      <c r="S217" s="15"/>
+      <c r="T217" s="15"/>
+      <c r="U217" s="15"/>
+    </row>
+    <row r="218" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A218" s="7"/>
       <c r="B218" s="11"/>
       <c r="C218" s="8"/>
@@ -7119,22 +7215,22 @@
       <c r="E218" s="8"/>
       <c r="F218" s="8"/>
       <c r="G218" s="8"/>
-      <c r="H218" s="16"/>
-      <c r="I218" s="30"/>
-      <c r="J218" s="30"/>
-      <c r="K218" s="30"/>
-      <c r="L218" s="30"/>
-      <c r="M218" s="43"/>
-      <c r="N218" s="43"/>
-      <c r="O218" s="16"/>
-      <c r="P218" s="16"/>
-      <c r="Q218" s="16"/>
-      <c r="R218" s="16"/>
-      <c r="S218" s="16"/>
-      <c r="T218" s="16"/>
-      <c r="U218" s="16"/>
-    </row>
-    <row r="219" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H218" s="15"/>
+      <c r="I218" s="29"/>
+      <c r="J218" s="29"/>
+      <c r="K218" s="29"/>
+      <c r="L218" s="29"/>
+      <c r="M218" s="42"/>
+      <c r="N218" s="42"/>
+      <c r="O218" s="15"/>
+      <c r="P218" s="15"/>
+      <c r="Q218" s="15"/>
+      <c r="R218" s="15"/>
+      <c r="S218" s="15"/>
+      <c r="T218" s="15"/>
+      <c r="U218" s="15"/>
+    </row>
+    <row r="219" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A219" s="7"/>
       <c r="B219" s="11"/>
       <c r="C219" s="8"/>
@@ -7142,22 +7238,22 @@
       <c r="E219" s="8"/>
       <c r="F219" s="8"/>
       <c r="G219" s="8"/>
-      <c r="H219" s="16"/>
-      <c r="I219" s="30"/>
-      <c r="J219" s="30"/>
-      <c r="K219" s="30"/>
-      <c r="L219" s="30"/>
-      <c r="M219" s="43"/>
-      <c r="N219" s="43"/>
-      <c r="O219" s="16"/>
-      <c r="P219" s="16"/>
-      <c r="Q219" s="16"/>
-      <c r="R219" s="16"/>
-      <c r="S219" s="16"/>
-      <c r="T219" s="16"/>
-      <c r="U219" s="16"/>
-    </row>
-    <row r="220" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H219" s="15"/>
+      <c r="I219" s="29"/>
+      <c r="J219" s="29"/>
+      <c r="K219" s="29"/>
+      <c r="L219" s="29"/>
+      <c r="M219" s="42"/>
+      <c r="N219" s="42"/>
+      <c r="O219" s="15"/>
+      <c r="P219" s="15"/>
+      <c r="Q219" s="15"/>
+      <c r="R219" s="15"/>
+      <c r="S219" s="15"/>
+      <c r="T219" s="15"/>
+      <c r="U219" s="15"/>
+    </row>
+    <row r="220" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A220" s="7"/>
       <c r="B220" s="11"/>
       <c r="C220" s="8"/>
@@ -7165,22 +7261,22 @@
       <c r="E220" s="8"/>
       <c r="F220" s="8"/>
       <c r="G220" s="8"/>
-      <c r="H220" s="16"/>
-      <c r="I220" s="30"/>
-      <c r="J220" s="30"/>
-      <c r="K220" s="30"/>
-      <c r="L220" s="30"/>
-      <c r="M220" s="43"/>
-      <c r="N220" s="43"/>
-      <c r="O220" s="16"/>
-      <c r="P220" s="16"/>
-      <c r="Q220" s="16"/>
-      <c r="R220" s="16"/>
-      <c r="S220" s="16"/>
-      <c r="T220" s="16"/>
-      <c r="U220" s="16"/>
-    </row>
-    <row r="221" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H220" s="15"/>
+      <c r="I220" s="29"/>
+      <c r="J220" s="29"/>
+      <c r="K220" s="29"/>
+      <c r="L220" s="29"/>
+      <c r="M220" s="42"/>
+      <c r="N220" s="42"/>
+      <c r="O220" s="15"/>
+      <c r="P220" s="15"/>
+      <c r="Q220" s="15"/>
+      <c r="R220" s="15"/>
+      <c r="S220" s="15"/>
+      <c r="T220" s="15"/>
+      <c r="U220" s="15"/>
+    </row>
+    <row r="221" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A221" s="7"/>
       <c r="B221" s="11"/>
       <c r="C221" s="8"/>
@@ -7188,22 +7284,22 @@
       <c r="E221" s="8"/>
       <c r="F221" s="8"/>
       <c r="G221" s="8"/>
-      <c r="H221" s="16"/>
-      <c r="I221" s="30"/>
-      <c r="J221" s="30"/>
-      <c r="K221" s="30"/>
-      <c r="L221" s="30"/>
-      <c r="M221" s="43"/>
-      <c r="N221" s="43"/>
-      <c r="O221" s="16"/>
-      <c r="P221" s="16"/>
-      <c r="Q221" s="16"/>
-      <c r="R221" s="16"/>
-      <c r="S221" s="16"/>
-      <c r="T221" s="16"/>
-      <c r="U221" s="16"/>
-    </row>
-    <row r="222" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H221" s="15"/>
+      <c r="I221" s="29"/>
+      <c r="J221" s="29"/>
+      <c r="K221" s="29"/>
+      <c r="L221" s="29"/>
+      <c r="M221" s="42"/>
+      <c r="N221" s="42"/>
+      <c r="O221" s="15"/>
+      <c r="P221" s="15"/>
+      <c r="Q221" s="15"/>
+      <c r="R221" s="15"/>
+      <c r="S221" s="15"/>
+      <c r="T221" s="15"/>
+      <c r="U221" s="15"/>
+    </row>
+    <row r="222" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A222" s="7"/>
       <c r="B222" s="11"/>
       <c r="C222" s="8"/>
@@ -7211,22 +7307,22 @@
       <c r="E222" s="8"/>
       <c r="F222" s="8"/>
       <c r="G222" s="8"/>
-      <c r="H222" s="16"/>
-      <c r="I222" s="30"/>
-      <c r="J222" s="30"/>
-      <c r="K222" s="30"/>
-      <c r="L222" s="30"/>
-      <c r="M222" s="43"/>
-      <c r="N222" s="43"/>
-      <c r="O222" s="16"/>
-      <c r="P222" s="16"/>
-      <c r="Q222" s="16"/>
-      <c r="R222" s="16"/>
-      <c r="S222" s="16"/>
-      <c r="T222" s="16"/>
-      <c r="U222" s="16"/>
-    </row>
-    <row r="223" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H222" s="15"/>
+      <c r="I222" s="29"/>
+      <c r="J222" s="29"/>
+      <c r="K222" s="29"/>
+      <c r="L222" s="29"/>
+      <c r="M222" s="42"/>
+      <c r="N222" s="42"/>
+      <c r="O222" s="15"/>
+      <c r="P222" s="15"/>
+      <c r="Q222" s="15"/>
+      <c r="R222" s="15"/>
+      <c r="S222" s="15"/>
+      <c r="T222" s="15"/>
+      <c r="U222" s="15"/>
+    </row>
+    <row r="223" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A223" s="7"/>
       <c r="B223" s="11"/>
       <c r="C223" s="8"/>
@@ -7234,20 +7330,20 @@
       <c r="E223" s="8"/>
       <c r="F223" s="8"/>
       <c r="G223" s="8"/>
-      <c r="H223" s="16"/>
-      <c r="I223" s="30"/>
-      <c r="J223" s="30"/>
-      <c r="K223" s="30"/>
-      <c r="L223" s="30"/>
-      <c r="M223" s="43"/>
-      <c r="N223" s="43"/>
-      <c r="O223" s="16"/>
-      <c r="P223" s="16"/>
-      <c r="Q223" s="16"/>
-      <c r="R223" s="16"/>
-      <c r="S223" s="16"/>
-      <c r="T223" s="16"/>
-      <c r="U223" s="16"/>
+      <c r="H223" s="15"/>
+      <c r="I223" s="29"/>
+      <c r="J223" s="29"/>
+      <c r="K223" s="29"/>
+      <c r="L223" s="29"/>
+      <c r="M223" s="42"/>
+      <c r="N223" s="42"/>
+      <c r="O223" s="15"/>
+      <c r="P223" s="15"/>
+      <c r="Q223" s="15"/>
+      <c r="R223" s="15"/>
+      <c r="S223" s="15"/>
+      <c r="T223" s="15"/>
+      <c r="U223" s="15"/>
     </row>
     <row r="224" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B224" s="11"/>
@@ -8553,6 +8649,9 @@
     <hyperlink ref="B76" r:id="rId2" location="ci-c-spec-35" xr:uid="{5FF64713-34D9-A748-A286-5A4D61DB8334}"/>
     <hyperlink ref="B52" r:id="rId3" location="ci-c-spec-11" xr:uid="{4E0F9A5A-0897-2C4B-98E8-127D0E73D6C1}"/>
     <hyperlink ref="B106" r:id="rId4" location="ci-c-spec-65" xr:uid="{2C76CA9A-AF34-C946-9996-4CD6012F10C0}"/>
+    <hyperlink ref="B30" r:id="rId5" location="ci-c-prof-1" xr:uid="{A9C2EE33-F35E-F940-908E-4D2AC2C145D0}"/>
+    <hyperlink ref="B33" r:id="rId6" location="ci-c-prof-4" xr:uid="{3D08F4CD-6E58-F249-9D1F-82381F024DB4}"/>
+    <hyperlink ref="B88" r:id="rId7" location="ci-c-spec-47" xr:uid="{7A99DCFA-1009-2246-AEDC-698721C9B204}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
@@ -8588,96 +8687,96 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="56.5" style="19" customWidth="1"/>
+    <col min="2" max="2" width="56.5" style="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="49" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="50"/>
+      <c r="B1" s="49"/>
     </row>
     <row r="2" spans="1:2" ht="82" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="50"/>
-      <c r="B2" s="50"/>
+      <c r="A2" s="49"/>
+      <c r="B2" s="49"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="17" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="17" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="17" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="17" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="17" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="17" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="17" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="B13" s="40" t="s">
+      <c r="B13" s="39" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="85" x14ac:dyDescent="0.2">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="B14" s="41" t="s">
+      <c r="B14" s="40" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="136" x14ac:dyDescent="0.2">
-      <c r="B15" s="41" t="s">
+      <c r="B15" s="40" t="s">
         <v>55</v>
       </c>
     </row>
@@ -8703,19 +8802,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="17" t="s">
         <v>59</v>
       </c>
     </row>
@@ -8814,28 +8913,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="b5a44311-ed64-4a72-909f-c9dc6973bde2" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Description xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
-    <SortOrder xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC335ED7BB179244BF94A0DFE64544DC" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d3a0f66abe5d2a0564332877ab55d3f7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eebd8b74-b9de-41b2-9247-c010c4973c2b" xmlns:ns3="b7009bbd-f938-489b-a530-f05273710fff" xmlns:ns4="b5a44311-ed64-4a72-909f-c9dc6973bde2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ec7ca2ee893ff8a0f61d4046c6461645" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
@@ -9089,10 +9166,44 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="b5a44311-ed64-4a72-909f-c9dc6973bde2" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Description xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
+    <SortOrder xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84097F-5807-4DCF-92C6-48C9EE26CFB8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12FB330C-B068-4EE3-928A-A72A297ABA91}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
+    <ds:schemaRef ds:uri="b7009bbd-f938-489b-a530-f05273710fff"/>
+    <ds:schemaRef ds:uri="b5a44311-ed64-4a72-909f-c9dc6973bde2"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9116,21 +9227,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12FB330C-B068-4EE3-928A-A72A297ABA91}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84097F-5807-4DCF-92C6-48C9EE26CFB8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
-    <ds:schemaRef ds:uri="b7009bbd-f938-489b-a530-f05273710fff"/>
-    <ds:schemaRef ds:uri="b5a44311-ed64-4a72-909f-c9dc6973bde2"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update requirements mapping for client v2.2.1
</commit_message>
<xml_diff>
--- a/lib/davinci_pas_test_kit/requirements/hl7.fhir.us.davinci-pas_2.2.1_requirements.xlsx
+++ b/lib/davinci_pas_test_kit/requirements/hl7.fhir.us.davinci-pas_2.2.1_requirements.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karlnaden/GlenViewAssociates/Inferno/source/davinci-pas-test-kit/lib/davinci_pas_test_kit/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B3BEC42-E831-164D-B0D3-5BF7C2F1422B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8115E68B-45AF-3F43-9D3B-81B26D0AE85B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20100" activeTab="1" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
   </bookViews>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="770" uniqueCount="447">
   <si>
     <r>
       <rPr>
@@ -2706,39 +2706,33 @@
     <t>Attestation (maybe Mechanical piece- require incomplete responses - should happen naturally)</t>
   </si>
   <si>
+    <t>TODO</t>
+  </si>
+  <si>
+    <t>TODO - see CRD ID-119</t>
+  </si>
+  <si>
+    <t>Attestatation</t>
+  </si>
+  <si>
+    <t>?? Mechnical if possible</t>
+  </si>
+  <si>
+    <t>Wrong Actor - Mechnical</t>
+  </si>
+  <si>
     <t>Bundle.entry.fullUrl values **SHALL** be:
 - the URL at which the resource is available from the EHR if exposed via the client's REST interface; or
 - the form "urn:uuid:[some guid]"</t>
   </si>
   <si>
-    <t>ID-148</t>
-  </si>
-  <si>
-    <t>ID-150</t>
-  </si>
-  <si>
-    <t>Future</t>
-  </si>
-  <si>
-    <t>ID-56</t>
-  </si>
-  <si>
-    <t>Done - Double Check</t>
-  </si>
-  <si>
     <t>Done</t>
   </si>
   <si>
-    <t>ID-151</t>
-  </si>
-  <si>
-    <t>Actor adjusted payer -&gt; client</t>
-  </si>
-  <si>
-    <t>Actor adjusted client -&gt; payer</t>
-  </si>
-  <si>
-    <t>Actor adjusted client + payer -&gt; payer</t>
+    <t>Changed the Actor because the server is responsible for returning the OperationOutcome, not the client</t>
+  </si>
+  <si>
+    <t>Updated actor - Client is responsible for the Claim</t>
   </si>
 </sst>
 </file>
@@ -3138,7 +3132,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3155,6 +3149,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -3595,72 +3590,72 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="133.5" style="23" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" style="19"/>
-    <col min="3" max="3" width="91.1640625" style="19" customWidth="1"/>
-    <col min="4" max="16384" width="10.83203125" style="14"/>
+    <col min="1" max="1" width="133.5" style="24" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" style="20"/>
+    <col min="3" max="3" width="91.1640625" style="20" customWidth="1"/>
+    <col min="4" max="16384" width="10.83203125" style="15"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="340" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="24" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="32" t="s">
+      <c r="A1" s="25" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="33" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="124.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="36"/>
+      <c r="C2" s="37"/>
     </row>
     <row r="3" spans="1:3" ht="134" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="33"/>
+      <c r="C3" s="34"/>
     </row>
     <row r="4" spans="1:3" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="44" t="s">
+      <c r="A4" s="45" t="s">
         <v>69</v>
       </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="35"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="36"/>
     </row>
     <row r="5" spans="1:3" ht="258" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="45"/>
-      <c r="B5" s="38"/>
-      <c r="C5" s="33"/>
+      <c r="A5" s="46"/>
+      <c r="B5" s="39"/>
+      <c r="C5" s="34"/>
     </row>
     <row r="6" spans="1:3" ht="164" x14ac:dyDescent="0.2">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="26"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="27"/>
     </row>
     <row r="7" spans="1:3" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="46" t="s">
+      <c r="A7" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="47"/>
+      <c r="B7" s="48"/>
     </row>
     <row r="8" spans="1:3" ht="126" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="46"/>
-      <c r="B8" s="48"/>
+      <c r="A8" s="47"/>
+      <c r="B8" s="49"/>
     </row>
     <row r="9" spans="1:3" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="44"/>
-      <c r="B9" s="37"/>
+      <c r="A9" s="45"/>
+      <c r="B9" s="38"/>
     </row>
     <row r="10" spans="1:3" ht="292" x14ac:dyDescent="0.2">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="22" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="22"/>
+      <c r="A11" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3683,19 +3678,19 @@
     <col min="5" max="5" width="10.83203125" style="7"/>
     <col min="6" max="6" width="13.33203125" style="8" customWidth="1"/>
     <col min="7" max="7" width="14" style="7" customWidth="1"/>
-    <col min="8" max="8" width="24.6640625" style="15" customWidth="1"/>
-    <col min="9" max="9" width="10" style="29" customWidth="1"/>
-    <col min="10" max="10" width="22" style="29" customWidth="1"/>
-    <col min="11" max="11" width="10.5" style="29" customWidth="1"/>
-    <col min="12" max="12" width="25.83203125" style="29" customWidth="1"/>
+    <col min="8" max="8" width="24.6640625" style="16" customWidth="1"/>
+    <col min="9" max="9" width="10" style="30" customWidth="1"/>
+    <col min="10" max="10" width="22" style="30" customWidth="1"/>
+    <col min="11" max="11" width="10.5" style="30" customWidth="1"/>
+    <col min="12" max="12" width="25.83203125" style="30" customWidth="1"/>
     <col min="13" max="13" width="20" style="9" customWidth="1"/>
     <col min="14" max="14" width="28.5" style="9" customWidth="1"/>
     <col min="15" max="16" width="10.83203125" style="10" customWidth="1"/>
-    <col min="17" max="17" width="10.5" style="15" customWidth="1"/>
-    <col min="18" max="18" width="42.5" style="15" customWidth="1"/>
+    <col min="17" max="17" width="10.5" style="16" customWidth="1"/>
+    <col min="18" max="18" width="42.5" style="16" customWidth="1"/>
     <col min="19" max="19" width="15.83203125" style="10" customWidth="1"/>
     <col min="20" max="20" width="44.1640625" style="10" customWidth="1"/>
-    <col min="21" max="21" width="44.1640625" style="15" customWidth="1"/>
+    <col min="21" max="21" width="44.1640625" style="16" customWidth="1"/>
     <col min="22" max="23" width="10.83203125" style="6"/>
     <col min="24" max="24" width="14.83203125" style="6" customWidth="1"/>
     <col min="25" max="16384" width="10.83203125" style="6"/>
@@ -3723,19 +3718,19 @@
       <c r="G1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="H1" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="31" t="s">
+      <c r="I1" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="J1" s="31" t="s">
+      <c r="J1" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="K1" s="31" t="s">
+      <c r="K1" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="L1" s="31" t="s">
+      <c r="L1" s="32" t="s">
         <v>17</v>
       </c>
       <c r="M1" s="3" t="s">
@@ -3750,19 +3745,19 @@
       <c r="P1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="Q1" s="16" t="s">
+      <c r="Q1" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="R1" s="16" t="s">
+      <c r="R1" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="S1" s="16" t="s">
+      <c r="S1" s="17" t="s">
         <v>431</v>
       </c>
       <c r="T1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="U1" s="16" t="s">
+      <c r="U1" s="17" t="s">
         <v>25</v>
       </c>
       <c r="Y1" s="6"/>
@@ -3790,11 +3785,11 @@
         <v>428</v>
       </c>
       <c r="R2" s="10"/>
-      <c r="Y2" s="12"/>
+      <c r="Y2" s="13"/>
       <c r="Z2" s="5"/>
       <c r="AA2" s="5"/>
       <c r="AB2" s="5"/>
-      <c r="AC2" s="12"/>
+      <c r="AC2" s="13"/>
       <c r="AD2" s="5"/>
       <c r="AE2" s="5"/>
       <c r="AG2" s="5"/>
@@ -3824,11 +3819,11 @@
         <v>428</v>
       </c>
       <c r="R3" s="10"/>
-      <c r="Y3" s="12"/>
+      <c r="Y3" s="13"/>
       <c r="Z3" s="5"/>
       <c r="AA3" s="5"/>
       <c r="AB3" s="5"/>
-      <c r="AC3" s="12"/>
+      <c r="AC3" s="13"/>
       <c r="AD3" s="5"/>
       <c r="AE3" s="5"/>
     </row>
@@ -3855,11 +3850,11 @@
         <v>428</v>
       </c>
       <c r="R4" s="10"/>
-      <c r="Y4" s="12"/>
+      <c r="Y4" s="13"/>
       <c r="Z4" s="5"/>
       <c r="AA4" s="5"/>
       <c r="AB4" s="5"/>
-      <c r="AC4" s="12"/>
+      <c r="AC4" s="13"/>
       <c r="AD4" s="5"/>
       <c r="AE4" s="5"/>
     </row>
@@ -3885,14 +3880,14 @@
       <c r="P5" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R5" s="15" t="s">
+      <c r="R5" s="16" t="s">
         <v>432</v>
       </c>
-      <c r="Y5" s="12"/>
+      <c r="Y5" s="13"/>
       <c r="Z5" s="5"/>
       <c r="AA5" s="5"/>
       <c r="AB5" s="5"/>
-      <c r="AC5" s="12"/>
+      <c r="AC5" s="13"/>
       <c r="AD5" s="5"/>
       <c r="AE5" s="5"/>
     </row>
@@ -3919,11 +3914,11 @@
         <v>428</v>
       </c>
       <c r="R6" s="10"/>
-      <c r="Y6" s="12"/>
+      <c r="Y6" s="13"/>
       <c r="Z6" s="5"/>
       <c r="AA6" s="5"/>
       <c r="AB6" s="5"/>
-      <c r="AC6" s="12"/>
+      <c r="AC6" s="13"/>
       <c r="AD6" s="5"/>
       <c r="AE6" s="5"/>
     </row>
@@ -3949,15 +3944,15 @@
       <c r="P7" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R7" s="15" t="s">
+      <c r="R7" s="16" t="s">
         <v>432</v>
       </c>
-      <c r="X7" s="13"/>
-      <c r="Y7" s="12"/>
+      <c r="X7" s="14"/>
+      <c r="Y7" s="13"/>
       <c r="Z7" s="5"/>
       <c r="AA7" s="5"/>
       <c r="AB7" s="5"/>
-      <c r="AC7" s="12"/>
+      <c r="AC7" s="13"/>
       <c r="AD7" s="5"/>
       <c r="AE7" s="5"/>
     </row>
@@ -3983,7 +3978,7 @@
       <c r="P8" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R8" s="15" t="s">
+      <c r="R8" s="16" t="s">
         <v>432</v>
       </c>
     </row>
@@ -4132,11 +4127,11 @@
       <c r="G15" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R15" s="15" t="s">
+      <c r="R15" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
     </row>
     <row r="16" spans="1:35" ht="51" x14ac:dyDescent="0.2">
@@ -4158,11 +4153,11 @@
       <c r="G16" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R16" s="15" t="s">
+      <c r="R16" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S16" s="10" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
     </row>
     <row r="17" spans="1:19" ht="51" x14ac:dyDescent="0.2">
@@ -4288,11 +4283,11 @@
       <c r="G22" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R22" s="15" t="s">
+      <c r="R22" s="16" t="s">
         <v>437</v>
       </c>
       <c r="S22" s="10" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="23" spans="1:19" ht="102" x14ac:dyDescent="0.2">
@@ -4314,11 +4309,11 @@
       <c r="G23" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R23" s="15" t="s">
+      <c r="R23" s="16" t="s">
         <v>435</v>
       </c>
       <c r="S23" s="10" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="24" spans="1:19" ht="136" x14ac:dyDescent="0.2">
@@ -4340,7 +4335,7 @@
       <c r="G24" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R24" s="15" t="s">
+      <c r="R24" s="16" t="s">
         <v>434</v>
       </c>
     </row>
@@ -4414,11 +4409,11 @@
       <c r="P27" s="10" t="s">
         <v>430</v>
       </c>
-      <c r="R27" s="15" t="s">
+      <c r="R27" s="16" t="s">
         <v>436</v>
       </c>
       <c r="S27" s="10" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="28" spans="1:19" ht="85" x14ac:dyDescent="0.2">
@@ -4491,11 +4486,11 @@
       <c r="P30" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R30" s="15" t="s">
+      <c r="R30" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S30" s="10" t="s">
-        <v>445</v>
+        <v>438</v>
       </c>
     </row>
     <row r="31" spans="1:19" ht="34" x14ac:dyDescent="0.2">
@@ -4520,11 +4515,11 @@
       <c r="P31" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R31" s="15" t="s">
+      <c r="R31" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S31" s="10" t="s">
-        <v>445</v>
+        <v>438</v>
       </c>
     </row>
     <row r="32" spans="1:19" ht="34" x14ac:dyDescent="0.2">
@@ -4546,11 +4541,11 @@
       <c r="G32" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R32" s="15" t="s">
+      <c r="R32" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S32" s="10" t="s">
-        <v>445</v>
+        <v>438</v>
       </c>
     </row>
     <row r="33" spans="1:19" ht="170" x14ac:dyDescent="0.2">
@@ -4575,11 +4570,11 @@
       <c r="P33" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R33" s="15" t="s">
+      <c r="R33" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S33" s="10" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="34" spans="1:19" ht="119" x14ac:dyDescent="0.2">
@@ -4604,11 +4599,11 @@
       <c r="P34" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R34" s="15" t="s">
+      <c r="R34" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S34" s="10" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="35" spans="1:19" ht="136" x14ac:dyDescent="0.2">
@@ -4633,11 +4628,11 @@
       <c r="P35" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R35" s="15" t="s">
+      <c r="R35" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S35" s="10" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="36" spans="1:19" ht="102" x14ac:dyDescent="0.2">
@@ -4662,11 +4657,11 @@
       <c r="P36" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R36" s="15" t="s">
+      <c r="R36" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S36" s="10" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="37" spans="1:19" ht="85" x14ac:dyDescent="0.2">
@@ -4691,11 +4686,11 @@
       <c r="P37" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R37" s="15" t="s">
+      <c r="R37" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S37" s="10" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="38" spans="1:19" ht="85" x14ac:dyDescent="0.2">
@@ -4720,11 +4715,11 @@
       <c r="P38" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R38" s="15" t="s">
+      <c r="R38" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S38" s="10" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="39" spans="1:19" ht="68" x14ac:dyDescent="0.2">
@@ -4749,11 +4744,11 @@
       <c r="P39" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="R39" s="15" t="s">
+      <c r="R39" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S39" s="10" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="40" spans="1:19" ht="85" x14ac:dyDescent="0.2">
@@ -4817,11 +4812,11 @@
       <c r="G42" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="R42" s="15" t="s">
+      <c r="R42" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S42" s="10" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="43" spans="1:19" ht="51" x14ac:dyDescent="0.2">
@@ -4885,11 +4880,11 @@
       <c r="G45" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="R45" s="15" t="s">
-        <v>436</v>
+      <c r="R45" s="16" t="s">
+        <v>440</v>
       </c>
       <c r="S45" s="10" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="46" spans="1:19" ht="68" x14ac:dyDescent="0.2">
@@ -4955,7 +4950,7 @@
       </c>
       <c r="R48" s="10"/>
     </row>
-    <row r="49" spans="1:21" ht="51" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="s">
         <v>167</v>
       </c>
@@ -4974,14 +4969,14 @@
       <c r="G49" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R49" s="15" t="s">
+      <c r="R49" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S49" s="10" t="s">
         <v>444</v>
       </c>
     </row>
-    <row r="50" spans="1:21" ht="102" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:19" ht="102" x14ac:dyDescent="0.2">
       <c r="A50" s="7" t="s">
         <v>169</v>
       </c>
@@ -5002,7 +4997,7 @@
       </c>
       <c r="R50" s="10"/>
     </row>
-    <row r="51" spans="1:21" ht="153" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:19" ht="153" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
         <v>171</v>
       </c>
@@ -5023,7 +5018,7 @@
       </c>
       <c r="R51" s="10"/>
     </row>
-    <row r="52" spans="1:21" ht="17" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:19" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="7" t="s">
         <v>173</v>
       </c>
@@ -5037,22 +5032,16 @@
         <v>26</v>
       </c>
       <c r="E52" s="7" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="G52" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R52" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S52" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="U52" s="15" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="53" spans="1:21" ht="102" x14ac:dyDescent="0.2">
+      <c r="R52" s="10" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="53" spans="1:19" ht="102" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
         <v>175</v>
       </c>
@@ -5066,22 +5055,16 @@
         <v>26</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="G53" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R53" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S53" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="U53" s="15" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="54" spans="1:21" ht="102" x14ac:dyDescent="0.2">
+      <c r="R53" s="10" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="54" spans="1:19" ht="102" x14ac:dyDescent="0.2">
       <c r="A54" s="7" t="s">
         <v>177</v>
       </c>
@@ -5095,22 +5078,16 @@
         <v>26</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="G54" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R54" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S54" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="U54" s="15" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="55" spans="1:21" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R54" s="10" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="55" spans="1:19" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
         <v>179</v>
       </c>
@@ -5124,22 +5101,16 @@
         <v>26</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="G55" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R55" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S55" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="U55" s="15" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="56" spans="1:21" ht="68" x14ac:dyDescent="0.2">
+      <c r="R55" s="10" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="56" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
         <v>181</v>
       </c>
@@ -5158,8 +5129,9 @@
       <c r="G56" s="7" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="57" spans="1:21" ht="85" x14ac:dyDescent="0.2">
+      <c r="R56" s="10"/>
+    </row>
+    <row r="57" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
         <v>183</v>
       </c>
@@ -5167,28 +5139,22 @@
         <v>184</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
       <c r="D57" s="7" t="s">
         <v>26</v>
       </c>
       <c r="E57" s="7" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="G57" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R57" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S57" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="U57" s="15" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="58" spans="1:21" ht="102" x14ac:dyDescent="0.2">
+      <c r="R57" s="10" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="58" spans="1:19" ht="102" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="s">
         <v>185</v>
       </c>
@@ -5202,22 +5168,16 @@
         <v>26</v>
       </c>
       <c r="E58" s="7" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="G58" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R58" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S58" s="10" t="s">
-        <v>443</v>
-      </c>
-      <c r="U58" s="15" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="59" spans="1:21" ht="68" x14ac:dyDescent="0.2">
+      <c r="R58" s="10" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="59" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A59" s="7" t="s">
         <v>187</v>
       </c>
@@ -5231,22 +5191,16 @@
         <v>26</v>
       </c>
       <c r="E59" s="7" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="G59" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R59" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S59" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="U59" s="15" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="60" spans="1:21" ht="51" x14ac:dyDescent="0.2">
+      <c r="R59" s="10" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="60" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A60" s="7" t="s">
         <v>189</v>
       </c>
@@ -5260,22 +5214,16 @@
         <v>26</v>
       </c>
       <c r="E60" s="7" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="G60" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R60" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S60" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="U60" s="15" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="61" spans="1:21" ht="68" x14ac:dyDescent="0.2">
+      <c r="R60" s="10" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="61" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A61" s="7" t="s">
         <v>191</v>
       </c>
@@ -5289,22 +5237,16 @@
         <v>26</v>
       </c>
       <c r="E61" s="7" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="G61" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R61" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S61" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="U61" s="15" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="62" spans="1:21" ht="51" x14ac:dyDescent="0.2">
+      <c r="R61" s="10" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="62" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A62" s="7" t="s">
         <v>193</v>
       </c>
@@ -5323,8 +5265,9 @@
       <c r="G62" s="7" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:21" ht="34" x14ac:dyDescent="0.2">
+      <c r="R62" s="10"/>
+    </row>
+    <row r="63" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
         <v>195</v>
       </c>
@@ -5338,22 +5281,16 @@
         <v>26</v>
       </c>
       <c r="E63" s="7" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="G63" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R63" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S63" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="U63" s="15" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="64" spans="1:21" ht="34" x14ac:dyDescent="0.2">
+      <c r="R63" s="10" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="64" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A64" s="7" t="s">
         <v>197</v>
       </c>
@@ -5367,19 +5304,13 @@
         <v>26</v>
       </c>
       <c r="E64" s="7" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="G64" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R64" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S64" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="U64" s="15" t="s">
-        <v>446</v>
+      <c r="R64" s="10" t="s">
+        <v>442</v>
       </c>
     </row>
     <row r="65" spans="1:21" ht="102" x14ac:dyDescent="0.2">
@@ -5438,16 +5369,13 @@
         <v>26</v>
       </c>
       <c r="E67" s="7" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="G67" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R67" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S67" s="10" t="s">
-        <v>444</v>
+      <c r="U67" s="16" t="s">
+        <v>445</v>
       </c>
     </row>
     <row r="68" spans="1:21" ht="51" x14ac:dyDescent="0.2">
@@ -5637,8 +5565,8 @@
       <c r="G76" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="U76" s="15" t="s">
-        <v>447</v>
+      <c r="U76" s="16" t="s">
+        <v>445</v>
       </c>
     </row>
     <row r="77" spans="1:21" ht="85" x14ac:dyDescent="0.2">
@@ -5725,7 +5653,7 @@
       </c>
       <c r="R80" s="10"/>
     </row>
-    <row r="81" spans="1:21" ht="68" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A81" s="7" t="s">
         <v>231</v>
       </c>
@@ -5746,7 +5674,7 @@
       </c>
       <c r="R81" s="10"/>
     </row>
-    <row r="82" spans="1:21" ht="51" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A82" s="7" t="s">
         <v>233</v>
       </c>
@@ -5767,7 +5695,7 @@
       </c>
       <c r="R82" s="10"/>
     </row>
-    <row r="83" spans="1:21" ht="68" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A83" s="7" t="s">
         <v>235</v>
       </c>
@@ -5788,7 +5716,7 @@
       </c>
       <c r="R83" s="10"/>
     </row>
-    <row r="84" spans="1:21" ht="34" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A84" s="7" t="s">
         <v>237</v>
       </c>
@@ -5809,7 +5737,7 @@
       </c>
       <c r="R84" s="10"/>
     </row>
-    <row r="85" spans="1:21" ht="68" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="s">
         <v>239</v>
       </c>
@@ -5830,7 +5758,7 @@
       </c>
       <c r="R85" s="10"/>
     </row>
-    <row r="86" spans="1:21" ht="68" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A86" s="7" t="s">
         <v>241</v>
       </c>
@@ -5851,7 +5779,7 @@
       </c>
       <c r="R86" s="10"/>
     </row>
-    <row r="87" spans="1:21" ht="68" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A87" s="7" t="s">
         <v>243</v>
       </c>
@@ -5872,7 +5800,7 @@
       </c>
       <c r="R87" s="10"/>
     </row>
-    <row r="88" spans="1:21" ht="136" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:19" ht="136" x14ac:dyDescent="0.2">
       <c r="A88" s="7" t="s">
         <v>245</v>
       </c>
@@ -5886,16 +5814,19 @@
         <v>26</v>
       </c>
       <c r="E88" s="7" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="G88" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="U88" s="15" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="89" spans="1:21" ht="85" x14ac:dyDescent="0.2">
+      <c r="R88" s="16" t="s">
+        <v>441</v>
+      </c>
+      <c r="S88" s="10" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="89" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A89" s="7" t="s">
         <v>247</v>
       </c>
@@ -5916,7 +5847,7 @@
       </c>
       <c r="R89" s="10"/>
     </row>
-    <row r="90" spans="1:21" ht="136" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:19" ht="136" x14ac:dyDescent="0.2">
       <c r="A90" s="7" t="s">
         <v>249</v>
       </c>
@@ -5937,7 +5868,7 @@
       </c>
       <c r="R90" s="10"/>
     </row>
-    <row r="91" spans="1:21" ht="102" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:19" ht="102" x14ac:dyDescent="0.2">
       <c r="A91" s="7" t="s">
         <v>251</v>
       </c>
@@ -5958,7 +5889,7 @@
       </c>
       <c r="R91" s="10"/>
     </row>
-    <row r="92" spans="1:21" ht="34" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A92" s="7" t="s">
         <v>253</v>
       </c>
@@ -5979,7 +5910,7 @@
       </c>
       <c r="R92" s="10"/>
     </row>
-    <row r="93" spans="1:21" ht="51" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A93" s="7" t="s">
         <v>255</v>
       </c>
@@ -6000,7 +5931,7 @@
       </c>
       <c r="R93" s="10"/>
     </row>
-    <row r="94" spans="1:21" ht="85" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A94" s="7" t="s">
         <v>257</v>
       </c>
@@ -6021,7 +5952,7 @@
       </c>
       <c r="R94" s="10"/>
     </row>
-    <row r="95" spans="1:21" ht="85" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A95" s="7" t="s">
         <v>259</v>
       </c>
@@ -6042,7 +5973,7 @@
       </c>
       <c r="R95" s="10"/>
     </row>
-    <row r="96" spans="1:21" ht="34" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A96" s="7" t="s">
         <v>261</v>
       </c>
@@ -6058,7 +5989,7 @@
       <c r="E96" s="7" t="s">
         <v>424</v>
       </c>
-      <c r="F96" s="28"/>
+      <c r="F96" s="29"/>
       <c r="G96" s="7" t="b">
         <v>0</v>
       </c>
@@ -6099,19 +6030,13 @@
         <v>26</v>
       </c>
       <c r="E98" s="7" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="G98" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R98" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S98" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="U98" s="15" t="s">
-        <v>446</v>
+      <c r="R98" s="10" t="s">
+        <v>442</v>
       </c>
     </row>
     <row r="99" spans="1:21" ht="34" x14ac:dyDescent="0.2">
@@ -6127,20 +6052,14 @@
       <c r="D99" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E99" s="7" t="s">
-        <v>425</v>
+      <c r="E99" s="12" t="s">
+        <v>424</v>
       </c>
       <c r="G99" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R99" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S99" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="U99" s="15" t="s">
-        <v>446</v>
+      <c r="R99" s="10" t="s">
+        <v>442</v>
       </c>
     </row>
     <row r="100" spans="1:21" ht="68" x14ac:dyDescent="0.2">
@@ -6225,7 +6144,7 @@
       <c r="G103" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R103" s="15" t="s">
+      <c r="R103" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S103" s="10" t="s">
@@ -6293,13 +6212,10 @@
       <c r="G106" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R106" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S106" s="10" t="s">
+      <c r="R106" s="10" t="s">
         <v>442</v>
       </c>
-      <c r="U106" s="15" t="s">
+      <c r="U106" s="16" t="s">
         <v>446</v>
       </c>
     </row>
@@ -6322,13 +6238,10 @@
       <c r="G107" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R107" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S107" s="10" t="s">
+      <c r="R107" s="10" t="s">
         <v>442</v>
       </c>
-      <c r="U107" s="15" t="s">
+      <c r="U107" s="16" t="s">
         <v>446</v>
       </c>
     </row>
@@ -6351,13 +6264,10 @@
       <c r="G108" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R108" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S108" s="10" t="s">
+      <c r="R108" s="10" t="s">
         <v>442</v>
       </c>
-      <c r="U108" s="15" t="s">
+      <c r="U108" s="16" t="s">
         <v>446</v>
       </c>
     </row>
@@ -6380,11 +6290,11 @@
       <c r="G109" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R109" s="15" t="s">
+      <c r="R109" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S109" s="10" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="110" spans="1:21" ht="119" x14ac:dyDescent="0.2">
@@ -6400,17 +6310,17 @@
       <c r="D110" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E110" s="41" t="s">
+      <c r="E110" s="42" t="s">
         <v>426</v>
       </c>
       <c r="G110" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R110" s="15" t="s">
+      <c r="R110" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S110" s="10" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="111" spans="1:21" ht="51" x14ac:dyDescent="0.2">
@@ -6426,17 +6336,17 @@
       <c r="D111" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E111" s="41" t="s">
+      <c r="E111" s="42" t="s">
         <v>426</v>
       </c>
       <c r="G111" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R111" s="15" t="s">
+      <c r="R111" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S111" s="10" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="112" spans="1:21" ht="119" x14ac:dyDescent="0.2">
@@ -6452,17 +6362,17 @@
       <c r="D112" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E112" s="41" t="s">
+      <c r="E112" s="42" t="s">
         <v>426</v>
       </c>
       <c r="G112" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R112" s="15" t="s">
+      <c r="R112" s="16" t="s">
         <v>433</v>
       </c>
       <c r="S112" s="10" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="113" spans="1:21" ht="102" x14ac:dyDescent="0.2">
@@ -6478,19 +6388,16 @@
       <c r="D113" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E113" s="7" t="s">
+      <c r="E113" s="42" t="s">
         <v>425</v>
       </c>
       <c r="G113" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="R113" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S113" s="10" t="s">
+      <c r="R113" s="10" t="s">
         <v>442</v>
       </c>
-      <c r="U113" s="15" t="s">
+      <c r="U113" s="16" t="s">
         <v>446</v>
       </c>
     </row>
@@ -6507,7 +6414,7 @@
       <c r="D114" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E114" s="41" t="s">
+      <c r="E114" s="42" t="s">
         <v>424</v>
       </c>
       <c r="G114" s="7" t="b">
@@ -6528,7 +6435,7 @@
       <c r="D115" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E115" s="41" t="s">
+      <c r="E115" s="42" t="s">
         <v>424</v>
       </c>
       <c r="G115" s="7" t="b">
@@ -6552,7 +6459,7 @@
       <c r="D116" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E116" s="41" t="s">
+      <c r="E116" s="42" t="s">
         <v>424</v>
       </c>
       <c r="G116" s="7" t="b">
@@ -6633,11 +6540,11 @@
       <c r="P119" s="10" t="s">
         <v>430</v>
       </c>
-      <c r="R119" s="15" t="s">
+      <c r="R119" s="16" t="s">
         <v>436</v>
       </c>
       <c r="S119" s="10" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="120" spans="1:21" ht="51" x14ac:dyDescent="0.2">
@@ -6674,16 +6581,16 @@
     </row>
     <row r="123" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B123" s="11"/>
-      <c r="I123" s="30"/>
-      <c r="J123" s="30"/>
-      <c r="K123" s="30"/>
-      <c r="L123" s="30"/>
+      <c r="I123" s="31"/>
+      <c r="J123" s="31"/>
+      <c r="K123" s="31"/>
+      <c r="L123" s="31"/>
       <c r="Q123" s="10"/>
       <c r="R123" s="10"/>
     </row>
     <row r="124" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B124" s="11"/>
-      <c r="E124" s="41"/>
+      <c r="E124" s="42"/>
       <c r="R124" s="10"/>
     </row>
     <row r="125" spans="1:21" ht="16" x14ac:dyDescent="0.2">
@@ -6704,42 +6611,42 @@
     </row>
     <row r="129" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B129" s="11"/>
-      <c r="E129" s="41"/>
+      <c r="E129" s="42"/>
       <c r="R129" s="10"/>
     </row>
     <row r="130" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B130" s="11"/>
-      <c r="E130" s="41"/>
+      <c r="E130" s="42"/>
       <c r="R130" s="10"/>
     </row>
     <row r="131" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B131" s="11"/>
-      <c r="E131" s="41"/>
+      <c r="E131" s="42"/>
       <c r="R131" s="10"/>
     </row>
     <row r="132" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B132" s="11"/>
-      <c r="E132" s="41"/>
+      <c r="E132" s="42"/>
       <c r="R132" s="10"/>
     </row>
     <row r="133" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B133" s="11"/>
-      <c r="E133" s="41"/>
+      <c r="E133" s="42"/>
       <c r="R133" s="10"/>
     </row>
     <row r="134" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B134" s="11"/>
-      <c r="E134" s="41"/>
+      <c r="E134" s="42"/>
       <c r="R134" s="10"/>
     </row>
     <row r="135" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B135" s="11"/>
-      <c r="E135" s="41"/>
+      <c r="E135" s="42"/>
       <c r="R135" s="10"/>
     </row>
     <row r="136" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B136" s="11"/>
-      <c r="E136" s="41"/>
+      <c r="E136" s="42"/>
       <c r="R136" s="10"/>
     </row>
     <row r="137" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6748,12 +6655,12 @@
     </row>
     <row r="138" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B138" s="11"/>
-      <c r="E138" s="41"/>
+      <c r="E138" s="42"/>
       <c r="R138" s="10"/>
     </row>
     <row r="139" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B139" s="11"/>
-      <c r="E139" s="41"/>
+      <c r="E139" s="42"/>
       <c r="R139" s="10"/>
     </row>
     <row r="140" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6762,7 +6669,7 @@
     </row>
     <row r="141" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B141" s="11"/>
-      <c r="E141" s="41"/>
+      <c r="E141" s="42"/>
       <c r="R141" s="10"/>
     </row>
     <row r="142" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6779,7 +6686,7 @@
     </row>
     <row r="145" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B145" s="11"/>
-      <c r="E145" s="41"/>
+      <c r="E145" s="42"/>
       <c r="R145" s="10"/>
     </row>
     <row r="146" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6788,32 +6695,32 @@
     </row>
     <row r="147" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B147" s="11"/>
-      <c r="E147" s="41"/>
+      <c r="E147" s="42"/>
       <c r="R147" s="10"/>
     </row>
     <row r="148" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B148" s="11"/>
-      <c r="E148" s="41"/>
+      <c r="E148" s="42"/>
       <c r="R148" s="10"/>
     </row>
     <row r="149" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B149" s="11"/>
-      <c r="E149" s="41"/>
+      <c r="E149" s="42"/>
       <c r="R149" s="10"/>
     </row>
     <row r="150" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B150" s="11"/>
-      <c r="E150" s="41"/>
+      <c r="E150" s="42"/>
       <c r="R150" s="10"/>
     </row>
     <row r="151" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B151" s="11"/>
-      <c r="E151" s="41"/>
+      <c r="E151" s="42"/>
       <c r="R151" s="10"/>
     </row>
     <row r="152" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B152" s="11"/>
-      <c r="E152" s="41"/>
+      <c r="E152" s="42"/>
       <c r="R152" s="10"/>
     </row>
     <row r="153" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6910,42 +6817,42 @@
     </row>
     <row r="176" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B176" s="11"/>
-      <c r="E176" s="41"/>
+      <c r="E176" s="42"/>
       <c r="R176" s="10"/>
     </row>
     <row r="177" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B177" s="11"/>
-      <c r="E177" s="41"/>
+      <c r="E177" s="42"/>
       <c r="R177" s="10"/>
     </row>
     <row r="178" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B178" s="11"/>
-      <c r="E178" s="41"/>
+      <c r="E178" s="42"/>
       <c r="R178" s="10"/>
     </row>
     <row r="179" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B179" s="11"/>
-      <c r="E179" s="41"/>
+      <c r="E179" s="42"/>
       <c r="R179" s="10"/>
     </row>
     <row r="180" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B180" s="11"/>
-      <c r="E180" s="41"/>
+      <c r="E180" s="42"/>
       <c r="R180" s="10"/>
     </row>
     <row r="181" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B181" s="11"/>
-      <c r="E181" s="41"/>
+      <c r="E181" s="42"/>
       <c r="R181" s="10"/>
     </row>
     <row r="182" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B182" s="11"/>
-      <c r="E182" s="41"/>
+      <c r="E182" s="42"/>
       <c r="R182" s="10"/>
     </row>
     <row r="183" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B183" s="11"/>
-      <c r="E183" s="41"/>
+      <c r="E183" s="42"/>
       <c r="R183" s="10"/>
     </row>
     <row r="184" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6954,7 +6861,7 @@
     </row>
     <row r="185" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B185" s="11"/>
-      <c r="E185" s="41"/>
+      <c r="E185" s="42"/>
       <c r="R185" s="10"/>
     </row>
     <row r="186" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6971,7 +6878,7 @@
     </row>
     <row r="189" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B189" s="11"/>
-      <c r="E189" s="41"/>
+      <c r="E189" s="42"/>
       <c r="R189" s="10"/>
     </row>
     <row r="190" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -6984,12 +6891,12 @@
     </row>
     <row r="192" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B192" s="11"/>
-      <c r="E192" s="41"/>
+      <c r="E192" s="42"/>
       <c r="R192" s="10"/>
     </row>
     <row r="193" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B193" s="11"/>
-      <c r="E193" s="41"/>
+      <c r="E193" s="42"/>
       <c r="R193" s="10"/>
     </row>
     <row r="194" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -7010,7 +6917,7 @@
     </row>
     <row r="198" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B198" s="11"/>
-      <c r="E198" s="41"/>
+      <c r="E198" s="42"/>
       <c r="R198" s="10"/>
     </row>
     <row r="199" spans="2:18" ht="16" x14ac:dyDescent="0.2">
@@ -7051,25 +6958,25 @@
     </row>
     <row r="208" spans="2:18" ht="16" x14ac:dyDescent="0.2">
       <c r="B208" s="11"/>
-      <c r="E208" s="41"/>
+      <c r="E208" s="42"/>
       <c r="R208" s="10"/>
     </row>
     <row r="209" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B209" s="11"/>
-      <c r="E209" s="41"/>
+      <c r="E209" s="42"/>
       <c r="R209" s="10"/>
     </row>
     <row r="210" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B210" s="11"/>
-      <c r="E210" s="41"/>
+      <c r="E210" s="42"/>
       <c r="R210" s="10"/>
     </row>
     <row r="211" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B211" s="11"/>
-      <c r="E211" s="41"/>
+      <c r="E211" s="42"/>
       <c r="R211" s="10"/>
     </row>
-    <row r="212" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A212" s="7"/>
       <c r="B212" s="11"/>
       <c r="C212" s="8"/>
@@ -7077,22 +6984,22 @@
       <c r="E212" s="8"/>
       <c r="F212" s="8"/>
       <c r="G212" s="8"/>
-      <c r="H212" s="15"/>
-      <c r="I212" s="29"/>
-      <c r="J212" s="29"/>
-      <c r="K212" s="29"/>
-      <c r="L212" s="29"/>
-      <c r="M212" s="42"/>
-      <c r="N212" s="42"/>
-      <c r="O212" s="15"/>
-      <c r="P212" s="15"/>
-      <c r="Q212" s="15"/>
-      <c r="R212" s="15"/>
-      <c r="S212" s="15"/>
-      <c r="T212" s="15"/>
-      <c r="U212" s="15"/>
-    </row>
-    <row r="213" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H212" s="16"/>
+      <c r="I212" s="30"/>
+      <c r="J212" s="30"/>
+      <c r="K212" s="30"/>
+      <c r="L212" s="30"/>
+      <c r="M212" s="43"/>
+      <c r="N212" s="43"/>
+      <c r="O212" s="16"/>
+      <c r="P212" s="16"/>
+      <c r="Q212" s="16"/>
+      <c r="R212" s="16"/>
+      <c r="S212" s="16"/>
+      <c r="T212" s="16"/>
+      <c r="U212" s="16"/>
+    </row>
+    <row r="213" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A213" s="7"/>
       <c r="B213" s="11"/>
       <c r="C213" s="8"/>
@@ -7100,22 +7007,22 @@
       <c r="E213" s="8"/>
       <c r="F213" s="8"/>
       <c r="G213" s="8"/>
-      <c r="H213" s="15"/>
-      <c r="I213" s="29"/>
-      <c r="J213" s="29"/>
-      <c r="K213" s="29"/>
-      <c r="L213" s="29"/>
-      <c r="M213" s="42"/>
-      <c r="N213" s="42"/>
-      <c r="O213" s="15"/>
-      <c r="P213" s="15"/>
-      <c r="Q213" s="15"/>
-      <c r="R213" s="15"/>
-      <c r="S213" s="15"/>
-      <c r="T213" s="15"/>
-      <c r="U213" s="15"/>
-    </row>
-    <row r="214" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H213" s="16"/>
+      <c r="I213" s="30"/>
+      <c r="J213" s="30"/>
+      <c r="K213" s="30"/>
+      <c r="L213" s="30"/>
+      <c r="M213" s="43"/>
+      <c r="N213" s="43"/>
+      <c r="O213" s="16"/>
+      <c r="P213" s="16"/>
+      <c r="Q213" s="16"/>
+      <c r="R213" s="16"/>
+      <c r="S213" s="16"/>
+      <c r="T213" s="16"/>
+      <c r="U213" s="16"/>
+    </row>
+    <row r="214" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A214" s="7"/>
       <c r="B214" s="11"/>
       <c r="C214" s="8"/>
@@ -7123,22 +7030,22 @@
       <c r="E214" s="8"/>
       <c r="F214" s="8"/>
       <c r="G214" s="8"/>
-      <c r="H214" s="15"/>
-      <c r="I214" s="29"/>
-      <c r="J214" s="29"/>
-      <c r="K214" s="29"/>
-      <c r="L214" s="29"/>
-      <c r="M214" s="42"/>
-      <c r="N214" s="42"/>
-      <c r="O214" s="15"/>
-      <c r="P214" s="15"/>
-      <c r="Q214" s="15"/>
-      <c r="R214" s="15"/>
-      <c r="S214" s="15"/>
-      <c r="T214" s="15"/>
-      <c r="U214" s="15"/>
-    </row>
-    <row r="215" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H214" s="16"/>
+      <c r="I214" s="30"/>
+      <c r="J214" s="30"/>
+      <c r="K214" s="30"/>
+      <c r="L214" s="30"/>
+      <c r="M214" s="43"/>
+      <c r="N214" s="43"/>
+      <c r="O214" s="16"/>
+      <c r="P214" s="16"/>
+      <c r="Q214" s="16"/>
+      <c r="R214" s="16"/>
+      <c r="S214" s="16"/>
+      <c r="T214" s="16"/>
+      <c r="U214" s="16"/>
+    </row>
+    <row r="215" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A215" s="7"/>
       <c r="B215" s="11"/>
       <c r="C215" s="8"/>
@@ -7146,22 +7053,22 @@
       <c r="E215" s="8"/>
       <c r="F215" s="8"/>
       <c r="G215" s="8"/>
-      <c r="H215" s="15"/>
-      <c r="I215" s="29"/>
-      <c r="J215" s="29"/>
-      <c r="K215" s="29"/>
-      <c r="L215" s="29"/>
-      <c r="M215" s="42"/>
-      <c r="N215" s="42"/>
-      <c r="O215" s="15"/>
-      <c r="P215" s="15"/>
-      <c r="Q215" s="15"/>
-      <c r="R215" s="15"/>
-      <c r="S215" s="15"/>
-      <c r="T215" s="15"/>
-      <c r="U215" s="15"/>
-    </row>
-    <row r="216" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H215" s="16"/>
+      <c r="I215" s="30"/>
+      <c r="J215" s="30"/>
+      <c r="K215" s="30"/>
+      <c r="L215" s="30"/>
+      <c r="M215" s="43"/>
+      <c r="N215" s="43"/>
+      <c r="O215" s="16"/>
+      <c r="P215" s="16"/>
+      <c r="Q215" s="16"/>
+      <c r="R215" s="16"/>
+      <c r="S215" s="16"/>
+      <c r="T215" s="16"/>
+      <c r="U215" s="16"/>
+    </row>
+    <row r="216" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A216" s="7"/>
       <c r="B216" s="11"/>
       <c r="C216" s="8"/>
@@ -7169,22 +7076,22 @@
       <c r="E216" s="8"/>
       <c r="F216" s="8"/>
       <c r="G216" s="8"/>
-      <c r="H216" s="15"/>
-      <c r="I216" s="29"/>
-      <c r="J216" s="29"/>
-      <c r="K216" s="29"/>
-      <c r="L216" s="29"/>
-      <c r="M216" s="42"/>
-      <c r="N216" s="42"/>
-      <c r="O216" s="15"/>
-      <c r="P216" s="15"/>
-      <c r="Q216" s="15"/>
-      <c r="R216" s="15"/>
-      <c r="S216" s="15"/>
-      <c r="T216" s="15"/>
-      <c r="U216" s="15"/>
-    </row>
-    <row r="217" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H216" s="16"/>
+      <c r="I216" s="30"/>
+      <c r="J216" s="30"/>
+      <c r="K216" s="30"/>
+      <c r="L216" s="30"/>
+      <c r="M216" s="43"/>
+      <c r="N216" s="43"/>
+      <c r="O216" s="16"/>
+      <c r="P216" s="16"/>
+      <c r="Q216" s="16"/>
+      <c r="R216" s="16"/>
+      <c r="S216" s="16"/>
+      <c r="T216" s="16"/>
+      <c r="U216" s="16"/>
+    </row>
+    <row r="217" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A217" s="7"/>
       <c r="B217" s="11"/>
       <c r="C217" s="8"/>
@@ -7192,22 +7099,22 @@
       <c r="E217" s="8"/>
       <c r="F217" s="8"/>
       <c r="G217" s="8"/>
-      <c r="H217" s="15"/>
-      <c r="I217" s="29"/>
-      <c r="J217" s="29"/>
-      <c r="K217" s="29"/>
-      <c r="L217" s="29"/>
-      <c r="M217" s="42"/>
-      <c r="N217" s="42"/>
-      <c r="O217" s="15"/>
-      <c r="P217" s="15"/>
-      <c r="Q217" s="15"/>
-      <c r="R217" s="15"/>
-      <c r="S217" s="15"/>
-      <c r="T217" s="15"/>
-      <c r="U217" s="15"/>
-    </row>
-    <row r="218" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H217" s="16"/>
+      <c r="I217" s="30"/>
+      <c r="J217" s="30"/>
+      <c r="K217" s="30"/>
+      <c r="L217" s="30"/>
+      <c r="M217" s="43"/>
+      <c r="N217" s="43"/>
+      <c r="O217" s="16"/>
+      <c r="P217" s="16"/>
+      <c r="Q217" s="16"/>
+      <c r="R217" s="16"/>
+      <c r="S217" s="16"/>
+      <c r="T217" s="16"/>
+      <c r="U217" s="16"/>
+    </row>
+    <row r="218" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A218" s="7"/>
       <c r="B218" s="11"/>
       <c r="C218" s="8"/>
@@ -7215,22 +7122,22 @@
       <c r="E218" s="8"/>
       <c r="F218" s="8"/>
       <c r="G218" s="8"/>
-      <c r="H218" s="15"/>
-      <c r="I218" s="29"/>
-      <c r="J218" s="29"/>
-      <c r="K218" s="29"/>
-      <c r="L218" s="29"/>
-      <c r="M218" s="42"/>
-      <c r="N218" s="42"/>
-      <c r="O218" s="15"/>
-      <c r="P218" s="15"/>
-      <c r="Q218" s="15"/>
-      <c r="R218" s="15"/>
-      <c r="S218" s="15"/>
-      <c r="T218" s="15"/>
-      <c r="U218" s="15"/>
-    </row>
-    <row r="219" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H218" s="16"/>
+      <c r="I218" s="30"/>
+      <c r="J218" s="30"/>
+      <c r="K218" s="30"/>
+      <c r="L218" s="30"/>
+      <c r="M218" s="43"/>
+      <c r="N218" s="43"/>
+      <c r="O218" s="16"/>
+      <c r="P218" s="16"/>
+      <c r="Q218" s="16"/>
+      <c r="R218" s="16"/>
+      <c r="S218" s="16"/>
+      <c r="T218" s="16"/>
+      <c r="U218" s="16"/>
+    </row>
+    <row r="219" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A219" s="7"/>
       <c r="B219" s="11"/>
       <c r="C219" s="8"/>
@@ -7238,22 +7145,22 @@
       <c r="E219" s="8"/>
       <c r="F219" s="8"/>
       <c r="G219" s="8"/>
-      <c r="H219" s="15"/>
-      <c r="I219" s="29"/>
-      <c r="J219" s="29"/>
-      <c r="K219" s="29"/>
-      <c r="L219" s="29"/>
-      <c r="M219" s="42"/>
-      <c r="N219" s="42"/>
-      <c r="O219" s="15"/>
-      <c r="P219" s="15"/>
-      <c r="Q219" s="15"/>
-      <c r="R219" s="15"/>
-      <c r="S219" s="15"/>
-      <c r="T219" s="15"/>
-      <c r="U219" s="15"/>
-    </row>
-    <row r="220" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H219" s="16"/>
+      <c r="I219" s="30"/>
+      <c r="J219" s="30"/>
+      <c r="K219" s="30"/>
+      <c r="L219" s="30"/>
+      <c r="M219" s="43"/>
+      <c r="N219" s="43"/>
+      <c r="O219" s="16"/>
+      <c r="P219" s="16"/>
+      <c r="Q219" s="16"/>
+      <c r="R219" s="16"/>
+      <c r="S219" s="16"/>
+      <c r="T219" s="16"/>
+      <c r="U219" s="16"/>
+    </row>
+    <row r="220" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A220" s="7"/>
       <c r="B220" s="11"/>
       <c r="C220" s="8"/>
@@ -7261,22 +7168,22 @@
       <c r="E220" s="8"/>
       <c r="F220" s="8"/>
       <c r="G220" s="8"/>
-      <c r="H220" s="15"/>
-      <c r="I220" s="29"/>
-      <c r="J220" s="29"/>
-      <c r="K220" s="29"/>
-      <c r="L220" s="29"/>
-      <c r="M220" s="42"/>
-      <c r="N220" s="42"/>
-      <c r="O220" s="15"/>
-      <c r="P220" s="15"/>
-      <c r="Q220" s="15"/>
-      <c r="R220" s="15"/>
-      <c r="S220" s="15"/>
-      <c r="T220" s="15"/>
-      <c r="U220" s="15"/>
-    </row>
-    <row r="221" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H220" s="16"/>
+      <c r="I220" s="30"/>
+      <c r="J220" s="30"/>
+      <c r="K220" s="30"/>
+      <c r="L220" s="30"/>
+      <c r="M220" s="43"/>
+      <c r="N220" s="43"/>
+      <c r="O220" s="16"/>
+      <c r="P220" s="16"/>
+      <c r="Q220" s="16"/>
+      <c r="R220" s="16"/>
+      <c r="S220" s="16"/>
+      <c r="T220" s="16"/>
+      <c r="U220" s="16"/>
+    </row>
+    <row r="221" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A221" s="7"/>
       <c r="B221" s="11"/>
       <c r="C221" s="8"/>
@@ -7284,22 +7191,22 @@
       <c r="E221" s="8"/>
       <c r="F221" s="8"/>
       <c r="G221" s="8"/>
-      <c r="H221" s="15"/>
-      <c r="I221" s="29"/>
-      <c r="J221" s="29"/>
-      <c r="K221" s="29"/>
-      <c r="L221" s="29"/>
-      <c r="M221" s="42"/>
-      <c r="N221" s="42"/>
-      <c r="O221" s="15"/>
-      <c r="P221" s="15"/>
-      <c r="Q221" s="15"/>
-      <c r="R221" s="15"/>
-      <c r="S221" s="15"/>
-      <c r="T221" s="15"/>
-      <c r="U221" s="15"/>
-    </row>
-    <row r="222" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H221" s="16"/>
+      <c r="I221" s="30"/>
+      <c r="J221" s="30"/>
+      <c r="K221" s="30"/>
+      <c r="L221" s="30"/>
+      <c r="M221" s="43"/>
+      <c r="N221" s="43"/>
+      <c r="O221" s="16"/>
+      <c r="P221" s="16"/>
+      <c r="Q221" s="16"/>
+      <c r="R221" s="16"/>
+      <c r="S221" s="16"/>
+      <c r="T221" s="16"/>
+      <c r="U221" s="16"/>
+    </row>
+    <row r="222" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A222" s="7"/>
       <c r="B222" s="11"/>
       <c r="C222" s="8"/>
@@ -7307,22 +7214,22 @@
       <c r="E222" s="8"/>
       <c r="F222" s="8"/>
       <c r="G222" s="8"/>
-      <c r="H222" s="15"/>
-      <c r="I222" s="29"/>
-      <c r="J222" s="29"/>
-      <c r="K222" s="29"/>
-      <c r="L222" s="29"/>
-      <c r="M222" s="42"/>
-      <c r="N222" s="42"/>
-      <c r="O222" s="15"/>
-      <c r="P222" s="15"/>
-      <c r="Q222" s="15"/>
-      <c r="R222" s="15"/>
-      <c r="S222" s="15"/>
-      <c r="T222" s="15"/>
-      <c r="U222" s="15"/>
-    </row>
-    <row r="223" spans="1:21" s="43" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="H222" s="16"/>
+      <c r="I222" s="30"/>
+      <c r="J222" s="30"/>
+      <c r="K222" s="30"/>
+      <c r="L222" s="30"/>
+      <c r="M222" s="43"/>
+      <c r="N222" s="43"/>
+      <c r="O222" s="16"/>
+      <c r="P222" s="16"/>
+      <c r="Q222" s="16"/>
+      <c r="R222" s="16"/>
+      <c r="S222" s="16"/>
+      <c r="T222" s="16"/>
+      <c r="U222" s="16"/>
+    </row>
+    <row r="223" spans="1:21" s="44" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A223" s="7"/>
       <c r="B223" s="11"/>
       <c r="C223" s="8"/>
@@ -7330,20 +7237,20 @@
       <c r="E223" s="8"/>
       <c r="F223" s="8"/>
       <c r="G223" s="8"/>
-      <c r="H223" s="15"/>
-      <c r="I223" s="29"/>
-      <c r="J223" s="29"/>
-      <c r="K223" s="29"/>
-      <c r="L223" s="29"/>
-      <c r="M223" s="42"/>
-      <c r="N223" s="42"/>
-      <c r="O223" s="15"/>
-      <c r="P223" s="15"/>
-      <c r="Q223" s="15"/>
-      <c r="R223" s="15"/>
-      <c r="S223" s="15"/>
-      <c r="T223" s="15"/>
-      <c r="U223" s="15"/>
+      <c r="H223" s="16"/>
+      <c r="I223" s="30"/>
+      <c r="J223" s="30"/>
+      <c r="K223" s="30"/>
+      <c r="L223" s="30"/>
+      <c r="M223" s="43"/>
+      <c r="N223" s="43"/>
+      <c r="O223" s="16"/>
+      <c r="P223" s="16"/>
+      <c r="Q223" s="16"/>
+      <c r="R223" s="16"/>
+      <c r="S223" s="16"/>
+      <c r="T223" s="16"/>
+      <c r="U223" s="16"/>
     </row>
     <row r="224" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="B224" s="11"/>
@@ -8649,9 +8556,7 @@
     <hyperlink ref="B76" r:id="rId2" location="ci-c-spec-35" xr:uid="{5FF64713-34D9-A748-A286-5A4D61DB8334}"/>
     <hyperlink ref="B52" r:id="rId3" location="ci-c-spec-11" xr:uid="{4E0F9A5A-0897-2C4B-98E8-127D0E73D6C1}"/>
     <hyperlink ref="B106" r:id="rId4" location="ci-c-spec-65" xr:uid="{2C76CA9A-AF34-C946-9996-4CD6012F10C0}"/>
-    <hyperlink ref="B30" r:id="rId5" location="ci-c-prof-1" xr:uid="{A9C2EE33-F35E-F940-908E-4D2AC2C145D0}"/>
-    <hyperlink ref="B33" r:id="rId6" location="ci-c-prof-4" xr:uid="{3D08F4CD-6E58-F249-9D1F-82381F024DB4}"/>
-    <hyperlink ref="B88" r:id="rId7" location="ci-c-spec-47" xr:uid="{7A99DCFA-1009-2246-AEDC-698721C9B204}"/>
+    <hyperlink ref="B67" r:id="rId5" location="ci-c-spec-26" xr:uid="{2791CF85-461B-1340-B643-634665A3629B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
@@ -8687,96 +8592,96 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="56.5" style="18" customWidth="1"/>
+    <col min="2" max="2" width="56.5" style="19" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="50" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="49"/>
+      <c r="B1" s="50"/>
     </row>
     <row r="2" spans="1:2" ht="82" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="49"/>
-      <c r="B2" s="49"/>
+      <c r="A2" s="50"/>
+      <c r="B2" s="50"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="18" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="18" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="18" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="18" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="18" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="18" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="18" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" s="17" t="s">
+      <c r="A13" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="B13" s="39" t="s">
+      <c r="B13" s="40" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="85" x14ac:dyDescent="0.2">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="B14" s="40" t="s">
+      <c r="B14" s="41" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="136" x14ac:dyDescent="0.2">
-      <c r="B15" s="40" t="s">
+      <c r="B15" s="41" t="s">
         <v>55</v>
       </c>
     </row>
@@ -8802,19 +8707,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="18" t="s">
         <v>59</v>
       </c>
     </row>

</xml_diff>